<commit_message>
Party indicator: switch to absentee-dashboard methodology
Replaces the 3-bucket LikelyParty split (large Unknown/Ind bucket) with the
dashboard rule used on absentee.vadems.org / cure.vadems.org: hard party ID,
then ND/U/I split by Clarity_DemSupport_26 at 50; only no-score/no-VAN is
Unknown (~2%). Two-way Dem/Rep is easier to read and consistent with the
dashboards.

Result (turnout = voted/Van-registered): Rep 53.0% vs Dem 45.1% (was 72.9/59.8
under 3-bucket); Democrats are the majority of voters (52.7% vs 45.4%),
consistent with Yes winning. Updates 5a/5e/5g, the exec summary, the HTML/PDF
brief + preview, and inventory notes.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -1038,58 +1038,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Dem</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>904974</v>
+        <v>1633612</v>
       </c>
       <c r="C2" t="n">
-        <v>1240690</v>
+        <v>3622724</v>
       </c>
       <c r="D2" t="n">
-        <v>72.90000000000001</v>
+        <v>45.1</v>
       </c>
       <c r="E2" t="n">
-        <v>29.2</v>
+        <v>52.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dem</t>
+          <t>Rep</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1276861</v>
+        <v>1409220</v>
       </c>
       <c r="C3" t="n">
-        <v>2135992</v>
+        <v>2659242</v>
       </c>
       <c r="D3" t="n">
-        <v>59.8</v>
+        <v>53</v>
       </c>
       <c r="E3" t="n">
-        <v>41.2</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Unknown/Ind</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>920077</v>
+        <v>59080</v>
       </c>
       <c r="C4" t="n">
-        <v>3009694</v>
+        <v>104410</v>
       </c>
       <c r="D4" t="n">
-        <v>30.6</v>
+        <v>56.6</v>
       </c>
       <c r="E4" t="n">
-        <v>29.7</v>
+        <v>1.9</v>
       </c>
     </row>
   </sheetData>
@@ -3591,11 +3591,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Unknown/Ind</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63973</v>
+        <v>26740</v>
       </c>
     </row>
     <row r="3">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>789</v>
+        <v>22082</v>
       </c>
     </row>
     <row r="4">
@@ -3615,7 +3615,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>132</v>
+        <v>16072</v>
       </c>
     </row>
   </sheetData>
@@ -4257,16 +4257,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>466681</v>
+        <v>557525</v>
       </c>
       <c r="C2" t="n">
-        <v>190098</v>
+        <v>229022</v>
       </c>
       <c r="D2" t="n">
-        <v>1830</v>
+        <v>2404</v>
       </c>
       <c r="E2" t="n">
-        <v>618252</v>
+        <v>844661</v>
       </c>
     </row>
     <row r="3">
@@ -4276,35 +4276,35 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>363524</v>
+        <v>505008</v>
       </c>
       <c r="C3" t="n">
-        <v>57110</v>
+        <v>85194</v>
       </c>
       <c r="D3" t="n">
-        <v>1112</v>
+        <v>1847</v>
       </c>
       <c r="E3" t="n">
-        <v>483228</v>
+        <v>817171</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Unknown/Ind</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>245920</v>
+        <v>13592</v>
       </c>
       <c r="C4" t="n">
-        <v>70026</v>
+        <v>3018</v>
       </c>
       <c r="D4" t="n">
-        <v>1378</v>
+        <v>69</v>
       </c>
       <c r="E4" t="n">
-        <v>602753</v>
+        <v>42401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add drop-off analysis (2025G voters who skipped the referendum)
#1 Analysis (aggregate, committed):
- New SQL table Historic.dbo.Dropoff_2025G_Base (2025G voters + voted_ref flag
  + age/sex/county/CD/party)
- analyze.py section 5i: drop-off by party, age, gender, CD, and county
  (top by count and by rate); xlsx sheets 5i_*; exec-summary finding #5
- Headline: 20.1% of 2025G voters dropped off; skewed young (42% of 18-24)
  and Democratic (22.3% vs 17.1% Rep)

#2 Targeting export (PII, NOT committed):
- export_dropoff_targets.py writes drop-off voter CSVs (VAN-ready) to
  C:\Absentee\Referendum2026_Dropoff_Targets\ (external). 690,881 voters +
  260,773 Dem-under-50 segment. .gitignore guards against committing voter files.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -20,6 +20,12 @@
     <sheet name="5f_weak_yes" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="5g_party" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="5h_precinct_anomalies" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="5i_dropoff_party" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="5i_dropoff_age" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="5i_dropoff_gender" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="5i_dropoff_cd" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="5i_dropoff_county_count" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="5i_dropoff_county_rate" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3567,6 +3573,990 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>party_bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1898003</v>
+      </c>
+      <c r="C2" t="n">
+        <v>423852</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1499364</v>
+      </c>
+      <c r="C3" t="n">
+        <v>256065</v>
+      </c>
+      <c r="D3" t="n">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>37517</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10964</v>
+      </c>
+      <c r="D4" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>age_band</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>215728</v>
+      </c>
+      <c r="C2" t="n">
+        <v>90516</v>
+      </c>
+      <c r="D2" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>386335</v>
+      </c>
+      <c r="C3" t="n">
+        <v>125803</v>
+      </c>
+      <c r="D3" t="n">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>507302</v>
+      </c>
+      <c r="C4" t="n">
+        <v>124584</v>
+      </c>
+      <c r="D4" t="n">
+        <v>24.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>549620</v>
+      </c>
+      <c r="C5" t="n">
+        <v>113205</v>
+      </c>
+      <c r="D5" t="n">
+        <v>20.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>666243</v>
+      </c>
+      <c r="C6" t="n">
+        <v>102423</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>636905</v>
+      </c>
+      <c r="C7" t="n">
+        <v>71222</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>472749</v>
+      </c>
+      <c r="C8" t="n">
+        <v>63128</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1563439</v>
+      </c>
+      <c r="C2" t="n">
+        <v>302556</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1865930</v>
+      </c>
+      <c r="C3" t="n">
+        <v>386420</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>396961</v>
+      </c>
+      <c r="C2" t="n">
+        <v>70343</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>312810</v>
+      </c>
+      <c r="C3" t="n">
+        <v>62387</v>
+      </c>
+      <c r="D3" t="n">
+        <v>19.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>239973</v>
+      </c>
+      <c r="C4" t="n">
+        <v>52758</v>
+      </c>
+      <c r="D4" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>307459</v>
+      </c>
+      <c r="C5" t="n">
+        <v>67475</v>
+      </c>
+      <c r="D5" t="n">
+        <v>21.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>345424</v>
+      </c>
+      <c r="C6" t="n">
+        <v>59746</v>
+      </c>
+      <c r="D6" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>309206</v>
+      </c>
+      <c r="C7" t="n">
+        <v>53522</v>
+      </c>
+      <c r="D7" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>302051</v>
+      </c>
+      <c r="C8" t="n">
+        <v>63427</v>
+      </c>
+      <c r="D8" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>300435</v>
+      </c>
+      <c r="C9" t="n">
+        <v>69842</v>
+      </c>
+      <c r="D9" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>290769</v>
+      </c>
+      <c r="C10" t="n">
+        <v>51804</v>
+      </c>
+      <c r="D10" t="n">
+        <v>17.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>311842</v>
+      </c>
+      <c r="C11" t="n">
+        <v>68094</v>
+      </c>
+      <c r="D11" t="n">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>317954</v>
+      </c>
+      <c r="C12" t="n">
+        <v>71483</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>locality</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fairfax</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>447400</v>
+      </c>
+      <c r="C2" t="n">
+        <v>101128</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Loudoun</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>169052</v>
+      </c>
+      <c r="C3" t="n">
+        <v>39141</v>
+      </c>
+      <c r="D3" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Prince William</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>166160</v>
+      </c>
+      <c r="C4" t="n">
+        <v>37715</v>
+      </c>
+      <c r="D4" t="n">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Virginia Beach (City)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>170015</v>
+      </c>
+      <c r="C5" t="n">
+        <v>36114</v>
+      </c>
+      <c r="D5" t="n">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>170654</v>
+      </c>
+      <c r="C6" t="n">
+        <v>33429</v>
+      </c>
+      <c r="D6" t="n">
+        <v>19.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Henrico</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>148965</v>
+      </c>
+      <c r="C7" t="n">
+        <v>30621</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>99732</v>
+      </c>
+      <c r="C8" t="n">
+        <v>23237</v>
+      </c>
+      <c r="D8" t="n">
+        <v>23.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Richmond (City)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>90278</v>
+      </c>
+      <c r="C9" t="n">
+        <v>21741</v>
+      </c>
+      <c r="D9" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Chesapeake (City)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>96441</v>
+      </c>
+      <c r="C10" t="n">
+        <v>19838</v>
+      </c>
+      <c r="D10" t="n">
+        <v>20.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alexandria (City)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>62937</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14991</v>
+      </c>
+      <c r="D11" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Norfolk (City)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>63595</v>
+      </c>
+      <c r="C12" t="n">
+        <v>14522</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Stafford</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>63319</v>
+      </c>
+      <c r="C13" t="n">
+        <v>13274</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>locality</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>g25_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dropped_off</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dropoff_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Harrisonburg (City)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>13087</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3702</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hopewell (City)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6662</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1674</v>
+      </c>
+      <c r="D3" t="n">
+        <v>25.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fredericksburg (City)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10562</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2637</v>
+      </c>
+      <c r="D4" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Charlottesville (City)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18516</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4464</v>
+      </c>
+      <c r="D5" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Richmond (City)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>90278</v>
+      </c>
+      <c r="C6" t="n">
+        <v>21741</v>
+      </c>
+      <c r="D6" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Petersburg (City)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10009</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2408</v>
+      </c>
+      <c r="D7" t="n">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Williamsburg (City)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6478</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1544</v>
+      </c>
+      <c r="D8" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alexandria (City)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>62937</v>
+      </c>
+      <c r="C9" t="n">
+        <v>14991</v>
+      </c>
+      <c r="D9" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Buchanan</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5423</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1291</v>
+      </c>
+      <c r="D10" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>99732</v>
+      </c>
+      <c r="C11" t="n">
+        <v>23237</v>
+      </c>
+      <c r="D11" t="n">
+        <v>23.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Loudoun</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>169052</v>
+      </c>
+      <c r="C12" t="n">
+        <v>39141</v>
+      </c>
+      <c r="D12" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>11092</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2545</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add surge analysis (5j) and one-page voter-churn brief
- analyze.py: new Surge_2026_Base table + section 5j (referendum voters who
  skipped 2025G), by party/age/gender/CD/county; xlsx sheets 5j_*
- Surge = 332,415 (10.8%), young, slightly Republican; net churn vs 2025G ~ -358k
- make_churn_brief.py + Referendum2026_Churn_Brief.{html,pdf,png}: one-page
  loss/gain brief (drop-off + surge), linked from README
- ignore __pycache__/*.pyc

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -26,6 +26,11 @@
     <sheet name="5i_dropoff_cd" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="5i_dropoff_county_count" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="5i_dropoff_county_rate" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="5j_surge_party" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="5j_surge_age" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="5j_surge_gender" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="5j_surge_cd" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="5j_surge_county_count" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4613,6 +4618,762 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>party_bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1633612</v>
+      </c>
+      <c r="C2" t="n">
+        <v>159461</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1409220</v>
+      </c>
+      <c r="C3" t="n">
+        <v>165921</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>33586</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7033</v>
+      </c>
+      <c r="D4" t="n">
+        <v>20.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>age_band</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>166643</v>
+      </c>
+      <c r="C2" t="n">
+        <v>41431</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>315837</v>
+      </c>
+      <c r="C3" t="n">
+        <v>55305</v>
+      </c>
+      <c r="D3" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>441836</v>
+      </c>
+      <c r="C4" t="n">
+        <v>59118</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>490247</v>
+      </c>
+      <c r="C5" t="n">
+        <v>53832</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>618722</v>
+      </c>
+      <c r="C6" t="n">
+        <v>54902</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>605380</v>
+      </c>
+      <c r="C7" t="n">
+        <v>39697</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>435593</v>
+      </c>
+      <c r="C8" t="n">
+        <v>25972</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2160</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2158</v>
+      </c>
+      <c r="D9" t="n">
+        <v>99.90000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1417506</v>
+      </c>
+      <c r="C2" t="n">
+        <v>156623</v>
+      </c>
+      <c r="D2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1654723</v>
+      </c>
+      <c r="C3" t="n">
+        <v>175213</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>357830</v>
+      </c>
+      <c r="C2" t="n">
+        <v>31212</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>280742</v>
+      </c>
+      <c r="C3" t="n">
+        <v>30319</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>212185</v>
+      </c>
+      <c r="C4" t="n">
+        <v>24970</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>265510</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25526</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>320603</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34925</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>292170</v>
+      </c>
+      <c r="C7" t="n">
+        <v>36486</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>269849</v>
+      </c>
+      <c r="C8" t="n">
+        <v>31225</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>252038</v>
+      </c>
+      <c r="C9" t="n">
+        <v>21445</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>278028</v>
+      </c>
+      <c r="C10" t="n">
+        <v>39063</v>
+      </c>
+      <c r="D10" t="n">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>274224</v>
+      </c>
+      <c r="C11" t="n">
+        <v>30476</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>273239</v>
+      </c>
+      <c r="C12" t="n">
+        <v>26768</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>locality</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fairfax</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>383154</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36882</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Prince William</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>145697</v>
+      </c>
+      <c r="C3" t="n">
+        <v>17252</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Loudoun</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>146585</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16674</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Virginia Beach (City)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>150106</v>
+      </c>
+      <c r="C5" t="n">
+        <v>16205</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>150578</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13353</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Henrico</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>128979</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10635</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chesapeake (City)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>86216</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9613</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>83257</v>
+      </c>
+      <c r="C9" t="n">
+        <v>6762</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Norfolk (City)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>55646</v>
+      </c>
+      <c r="C10" t="n">
+        <v>6573</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Richmond (City)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>74859</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6322</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spotsylvania</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>54521</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6304</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Newport News (City)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>50574</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6265</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add age x party cross-tabs to churn analysis + grouped brief charts
- analyze.py: §5i/§5j now include age x party drop-off/surge rate tables
  (Dem vs Rep within each age band + the gap); new xlsx sheets
  5i_dropoff_age_party, 5j_surge_age_party
- svg_grouped() accepts custom colors/gridstep
- churn brief: age charts are now grouped Dem-vs-Rep bars (drop-off & surge),
  replacing the separate age and party single-series charts; still one page
- Finding: Democrats drop off more than Republicans at every age band
  (widest at 18-24: ~45% vs ~37%); surge skews Republican at every age

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -26,11 +26,13 @@
     <sheet name="5i_dropoff_cd" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="5i_dropoff_county_count" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="5i_dropoff_county_rate" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="5j_surge_party" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="5j_surge_age" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="5j_surge_gender" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="5j_surge_cd" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="5j_surge_county_count" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="5i_dropoff_age_party" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="5j_surge_party" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="5j_surge_age" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="5j_surge_gender" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="5j_surge_cd" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="5j_surge_county_count" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="5j_surge_age_party" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4624,77 +4626,349 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>age_band</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>party_bucket</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>ref_voters</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>surge</t>
+          <t>g25</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>surge_pct</t>
+          <t>dropped</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Dem</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1633612</v>
-      </c>
       <c r="C2" t="n">
-        <v>159461</v>
+        <v>135237</v>
       </c>
       <c r="D2" t="n">
-        <v>9.800000000000001</v>
+        <v>60341</v>
+      </c>
+      <c r="E2" t="n">
+        <v>44.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Rep</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>1409220</v>
-      </c>
       <c r="C3" t="n">
-        <v>165921</v>
+        <v>74584</v>
       </c>
       <c r="D3" t="n">
-        <v>11.8</v>
+        <v>27622</v>
+      </c>
+      <c r="E3" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>247938</v>
+      </c>
+      <c r="D4" t="n">
+        <v>84927</v>
+      </c>
+      <c r="E4" t="n">
+        <v>34.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>131390</v>
+      </c>
+      <c r="D5" t="n">
+        <v>38322</v>
+      </c>
+      <c r="E5" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>309929</v>
+      </c>
+      <c r="D6" t="n">
+        <v>79336</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>191191</v>
+      </c>
+      <c r="D7" t="n">
+        <v>43347</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>312125</v>
+      </c>
+      <c r="D8" t="n">
+        <v>69044</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>232185</v>
+      </c>
+      <c r="D9" t="n">
+        <v>42764</v>
+      </c>
+      <c r="E9" t="n">
+        <v>18.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>334848</v>
+      </c>
+      <c r="D10" t="n">
+        <v>57441</v>
+      </c>
+      <c r="E10" t="n">
+        <v>17.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>325743</v>
+      </c>
+      <c r="D11" t="n">
+        <v>43781</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>323224</v>
+      </c>
+      <c r="D12" t="n">
+        <v>39898</v>
+      </c>
+      <c r="E12" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>308856</v>
+      </c>
+      <c r="D13" t="n">
+        <v>30497</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>234700</v>
+      </c>
+      <c r="D14" t="n">
+        <v>32865</v>
+      </c>
+      <c r="E14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>235415</v>
+      </c>
+      <c r="D15" t="n">
+        <v>29732</v>
+      </c>
+      <c r="E15" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>33586</v>
-      </c>
-      <c r="C4" t="n">
-        <v>7033</v>
-      </c>
-      <c r="D4" t="n">
-        <v>20.9</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4708,13 +4982,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>age_band</t>
+          <t>party_bucket</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -4736,129 +5010,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18-24</t>
+          <t>Dem</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166643</v>
+        <v>1633612</v>
       </c>
       <c r="C2" t="n">
-        <v>41431</v>
+        <v>159461</v>
       </c>
       <c r="D2" t="n">
-        <v>24.9</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25-34</t>
+          <t>Rep</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315837</v>
+        <v>1409220</v>
       </c>
       <c r="C3" t="n">
-        <v>55305</v>
+        <v>165921</v>
       </c>
       <c r="D3" t="n">
-        <v>17.5</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>35-44</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>441836</v>
+        <v>33586</v>
       </c>
       <c r="C4" t="n">
-        <v>59118</v>
+        <v>7033</v>
       </c>
       <c r="D4" t="n">
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>45-54</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>490247</v>
-      </c>
-      <c r="C5" t="n">
-        <v>53832</v>
-      </c>
-      <c r="D5" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>55-64</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>618722</v>
-      </c>
-      <c r="C6" t="n">
-        <v>54902</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>65-74</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>605380</v>
-      </c>
-      <c r="C7" t="n">
-        <v>39697</v>
-      </c>
-      <c r="D7" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>75+</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>435593</v>
-      </c>
-      <c r="C8" t="n">
-        <v>25972</v>
-      </c>
-      <c r="D8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2160</v>
-      </c>
-      <c r="C9" t="n">
-        <v>2158</v>
-      </c>
-      <c r="D9" t="n">
-        <v>99.90000000000001</v>
+        <v>20.9</v>
       </c>
     </row>
   </sheetData>
@@ -4872,13 +5066,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>age_band</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -4900,33 +5094,129 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>18-24</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1417506</v>
+        <v>166643</v>
       </c>
       <c r="C2" t="n">
-        <v>156623</v>
+        <v>41431</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>24.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>25-34</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1654723</v>
+        <v>315837</v>
       </c>
       <c r="C3" t="n">
-        <v>175213</v>
+        <v>55305</v>
       </c>
       <c r="D3" t="n">
-        <v>10.6</v>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>441836</v>
+      </c>
+      <c r="C4" t="n">
+        <v>59118</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>490247</v>
+      </c>
+      <c r="C5" t="n">
+        <v>53832</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>618722</v>
+      </c>
+      <c r="C6" t="n">
+        <v>54902</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>605380</v>
+      </c>
+      <c r="C7" t="n">
+        <v>39697</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>435593</v>
+      </c>
+      <c r="C8" t="n">
+        <v>25972</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2160</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2158</v>
+      </c>
+      <c r="D9" t="n">
+        <v>99.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -4940,13 +5230,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -4968,177 +5258,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>357830</v>
+        <v>1417506</v>
       </c>
       <c r="C2" t="n">
-        <v>31212</v>
+        <v>156623</v>
       </c>
       <c r="D2" t="n">
-        <v>8.699999999999999</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>280742</v>
+        <v>1654723</v>
       </c>
       <c r="C3" t="n">
-        <v>30319</v>
+        <v>175213</v>
       </c>
       <c r="D3" t="n">
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>212185</v>
-      </c>
-      <c r="C4" t="n">
-        <v>24970</v>
-      </c>
-      <c r="D4" t="n">
-        <v>11.8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>004</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>265510</v>
-      </c>
-      <c r="C5" t="n">
-        <v>25526</v>
-      </c>
-      <c r="D5" t="n">
-        <v>9.6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>005</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>320603</v>
-      </c>
-      <c r="C6" t="n">
-        <v>34925</v>
-      </c>
-      <c r="D6" t="n">
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>292170</v>
-      </c>
-      <c r="C7" t="n">
-        <v>36486</v>
-      </c>
-      <c r="D7" t="n">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>007</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>269849</v>
-      </c>
-      <c r="C8" t="n">
-        <v>31225</v>
-      </c>
-      <c r="D8" t="n">
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>008</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>252038</v>
-      </c>
-      <c r="C9" t="n">
-        <v>21445</v>
-      </c>
-      <c r="D9" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>009</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>278028</v>
-      </c>
-      <c r="C10" t="n">
-        <v>39063</v>
-      </c>
-      <c r="D10" t="n">
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>010</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>274224</v>
-      </c>
-      <c r="C11" t="n">
-        <v>30476</v>
-      </c>
-      <c r="D11" t="n">
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>011</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>273239</v>
-      </c>
-      <c r="C12" t="n">
-        <v>26768</v>
-      </c>
-      <c r="D12" t="n">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
     </row>
   </sheetData>
@@ -5152,6 +5298,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>357830</v>
+      </c>
+      <c r="C2" t="n">
+        <v>31212</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>280742</v>
+      </c>
+      <c r="C3" t="n">
+        <v>30319</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>212185</v>
+      </c>
+      <c r="C4" t="n">
+        <v>24970</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>265510</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25526</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>320603</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34925</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>292170</v>
+      </c>
+      <c r="C7" t="n">
+        <v>36486</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>269849</v>
+      </c>
+      <c r="C8" t="n">
+        <v>31225</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>252038</v>
+      </c>
+      <c r="C9" t="n">
+        <v>21445</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>278028</v>
+      </c>
+      <c r="C10" t="n">
+        <v>39063</v>
+      </c>
+      <c r="D10" t="n">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>274224</v>
+      </c>
+      <c r="C11" t="n">
+        <v>30476</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>273239</v>
+      </c>
+      <c r="C12" t="n">
+        <v>26768</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -5367,6 +5725,383 @@
       </c>
       <c r="D13" t="n">
         <v>12.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>age_band</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>party_bucket</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>refv</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>96641</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21745</v>
+      </c>
+      <c r="E2" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>65350</v>
+      </c>
+      <c r="D3" t="n">
+        <v>18388</v>
+      </c>
+      <c r="E3" t="n">
+        <v>28.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>190374</v>
+      </c>
+      <c r="D4" t="n">
+        <v>27363</v>
+      </c>
+      <c r="E4" t="n">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>119543</v>
+      </c>
+      <c r="D5" t="n">
+        <v>26475</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>259795</v>
+      </c>
+      <c r="D6" t="n">
+        <v>29202</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>176526</v>
+      </c>
+      <c r="D7" t="n">
+        <v>28682</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>268647</v>
+      </c>
+      <c r="D8" t="n">
+        <v>25566</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>216755</v>
+      </c>
+      <c r="D9" t="n">
+        <v>27334</v>
+      </c>
+      <c r="E9" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>301690</v>
+      </c>
+      <c r="D10" t="n">
+        <v>24283</v>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>311627</v>
+      </c>
+      <c r="D11" t="n">
+        <v>29665</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>301687</v>
+      </c>
+      <c r="D12" t="n">
+        <v>18361</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>298970</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20611</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>213515</v>
+      </c>
+      <c r="D14" t="n">
+        <v>11680</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>219647</v>
+      </c>
+      <c r="D15" t="n">
+        <v>13964</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1263</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1261</v>
+      </c>
+      <c r="E16" t="n">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>802</v>
+      </c>
+      <c r="D17" t="n">
+        <v>802</v>
+      </c>
+      <c r="E17" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Break top-locality drop-off chart into Dem vs Rep
- analyze.py §5i: new sheet 5i_dropoff_county_party + report table (top 12
  localities by drop-off count split by party)
- churn brief: locality chart is now grouped Dem-vs-Rep with value labels;
  finding notes the lost volume is overwhelmingly Democratic in the cities
  (Fairfax ~81k Dem vs ~19k Rep)
- svg_grouped: tolerate non-integer ymax

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -26,13 +26,14 @@
     <sheet name="5i_dropoff_cd" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="5i_dropoff_county_count" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="5i_dropoff_county_rate" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="5i_dropoff_age_party" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="5j_surge_party" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="5j_surge_age" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="5j_surge_gender" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="5j_surge_cd" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="5j_surge_county_count" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="5j_surge_age_party" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="5i_dropoff_county_party" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="5i_dropoff_age_party" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="5j_surge_party" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="5j_surge_age" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="5j_surge_gender" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="5j_surge_cd" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="5j_surge_county_count" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="5j_surge_age_party" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4626,349 +4627,2157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>age_band</t>
+          <t>locality</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>party_bucket</t>
+          <t>Dem</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>g25</t>
+          <t>Rep</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>dropped</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>rate</t>
+          <t>total</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18-24</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Fairfax</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>80994</v>
       </c>
       <c r="C2" t="n">
-        <v>135237</v>
+        <v>18911</v>
       </c>
       <c r="D2" t="n">
-        <v>60341</v>
-      </c>
-      <c r="E2" t="n">
-        <v>44.6</v>
+        <v>99905</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18-24</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Loudoun</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>25684</v>
       </c>
       <c r="C3" t="n">
-        <v>74584</v>
+        <v>12959</v>
       </c>
       <c r="D3" t="n">
-        <v>27622</v>
-      </c>
-      <c r="E3" t="n">
-        <v>37</v>
+        <v>38643</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25-34</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Prince William</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>26782</v>
       </c>
       <c r="C4" t="n">
-        <v>247938</v>
+        <v>10591</v>
       </c>
       <c r="D4" t="n">
-        <v>84927</v>
-      </c>
-      <c r="E4" t="n">
-        <v>34.3</v>
+        <v>37373</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25-34</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Virginia Beach (City)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>19919</v>
       </c>
       <c r="C5" t="n">
-        <v>131390</v>
+        <v>15660</v>
       </c>
       <c r="D5" t="n">
-        <v>38322</v>
-      </c>
-      <c r="E5" t="n">
-        <v>29.2</v>
+        <v>35579</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>35-44</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20565</v>
       </c>
       <c r="C6" t="n">
-        <v>309929</v>
+        <v>12467</v>
       </c>
       <c r="D6" t="n">
-        <v>79336</v>
-      </c>
-      <c r="E6" t="n">
-        <v>25.6</v>
+        <v>33032</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>35-44</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Henrico</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>22273</v>
       </c>
       <c r="C7" t="n">
-        <v>191191</v>
+        <v>7984</v>
       </c>
       <c r="D7" t="n">
-        <v>43347</v>
-      </c>
-      <c r="E7" t="n">
-        <v>22.7</v>
+        <v>30257</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>45-54</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20290</v>
       </c>
       <c r="C8" t="n">
-        <v>312125</v>
+        <v>2580</v>
       </c>
       <c r="D8" t="n">
-        <v>69044</v>
-      </c>
-      <c r="E8" t="n">
-        <v>22.1</v>
+        <v>22870</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>45-54</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Richmond (City)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>19326</v>
       </c>
       <c r="C9" t="n">
-        <v>232185</v>
+        <v>2009</v>
       </c>
       <c r="D9" t="n">
-        <v>42764</v>
-      </c>
-      <c r="E9" t="n">
-        <v>18.4</v>
+        <v>21335</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>55-64</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Chesapeake (City)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10973</v>
       </c>
       <c r="C10" t="n">
-        <v>334848</v>
+        <v>8549</v>
       </c>
       <c r="D10" t="n">
-        <v>57441</v>
-      </c>
-      <c r="E10" t="n">
-        <v>17.2</v>
+        <v>19522</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>55-64</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Alexandria (City)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>12980</v>
       </c>
       <c r="C11" t="n">
-        <v>325743</v>
+        <v>1740</v>
       </c>
       <c r="D11" t="n">
-        <v>43781</v>
-      </c>
-      <c r="E11" t="n">
-        <v>13.4</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>65-74</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Norfolk (City)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11977</v>
       </c>
       <c r="C12" t="n">
-        <v>323224</v>
+        <v>2329</v>
       </c>
       <c r="D12" t="n">
-        <v>39898</v>
-      </c>
-      <c r="E12" t="n">
-        <v>12.3</v>
+        <v>14306</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>65-74</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Stafford</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>7353</v>
       </c>
       <c r="C13" t="n">
-        <v>308856</v>
+        <v>5739</v>
       </c>
       <c r="D13" t="n">
-        <v>30497</v>
-      </c>
-      <c r="E13" t="n">
-        <v>9.9</v>
+        <v>13092</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>75+</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Newport News (City)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>9199</v>
       </c>
       <c r="C14" t="n">
-        <v>234700</v>
+        <v>2831</v>
       </c>
       <c r="D14" t="n">
-        <v>32865</v>
-      </c>
-      <c r="E14" t="n">
-        <v>14</v>
+        <v>12030</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>75+</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Rep</t>
-        </is>
+          <t>Spotsylvania</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5611</v>
       </c>
       <c r="C15" t="n">
-        <v>235415</v>
+        <v>5923</v>
       </c>
       <c r="D15" t="n">
-        <v>29732</v>
-      </c>
-      <c r="E15" t="n">
-        <v>12.6</v>
+        <v>11534</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Dem</t>
-        </is>
+          <t>Albemarle</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7857</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>2410</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
+        <v>10267</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hampton (City)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7909</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1648</v>
+      </c>
+      <c r="D17" t="n">
+        <v>9557</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hanover</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3131</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6129</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9260</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Montgomery</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5203</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2909</v>
+      </c>
+      <c r="D19" t="n">
+        <v>8112</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Suffolk (City)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5206</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2730</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7936</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Roanoke</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2559</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4559</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7118</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Portsmouth (City)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5668</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1405</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7073</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>James City</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3780</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3255</v>
+      </c>
+      <c r="D23" t="n">
+        <v>7035</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Roanoke (City)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4631</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2044</v>
+      </c>
+      <c r="D24" t="n">
+        <v>6675</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Frederick</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2117</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4484</v>
+      </c>
+      <c r="D25" t="n">
+        <v>6601</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fauquier</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2190</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3754</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5944</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lynchburg (City)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2437</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3170</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5607</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Bedford</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1179</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4218</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5397</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>York</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2517</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2625</v>
+      </c>
+      <c r="D29" t="n">
+        <v>5142</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Rockingham</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1396</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3402</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4798</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3563</v>
+      </c>
+      <c r="D31" t="n">
+        <v>4596</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Charlottesville (City)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4037</v>
+      </c>
+      <c r="C32" t="n">
+        <v>336</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4373</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Culpeper</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2564</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4217</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Campbell</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>955</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2943</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3898</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Harrisonburg (City)</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3031</v>
+      </c>
+      <c r="C35" t="n">
+        <v>578</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3609</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>781</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2740</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3521</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Pittsylvania</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1132</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2354</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3486</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Franklin</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>909</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2269</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3178</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Louisa</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1090</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1999</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3089</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Henry</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1173</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1848</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3021</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1067</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1903</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2970</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Isle of Wight</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1133</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1791</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2924</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Caroline</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1374</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2682</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Gloucester</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>739</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1907</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2646</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Manassas (City)</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1851</v>
+      </c>
+      <c r="C45" t="n">
+        <v>780</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2631</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Fredericksburg (City)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2065</v>
+      </c>
+      <c r="C46" t="n">
+        <v>545</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Warren</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>798</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1803</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2601</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sussex</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1451</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1138</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Shenandoah</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>657</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1930</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2587</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Powhatan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>601</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1945</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2546</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Danville (City)</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C51" t="n">
+        <v>690</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2534</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Goochland</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>989</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1517</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Wise</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>497</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1935</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Petersburg (City)</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2247</v>
+      </c>
+      <c r="C54" t="n">
+        <v>132</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Prince George</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1054</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1316</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2370</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>New Kent</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>722</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1536</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Fairfax (City)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1823</v>
+      </c>
+      <c r="C57" t="n">
+        <v>420</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Dinwiddie</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>954</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1283</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Accomack</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>989</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1216</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Botetourt</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>537</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1660</v>
+      </c>
+      <c r="D60" t="n">
+        <v>2197</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Fluvanna</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>951</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1223</v>
+      </c>
+      <c r="D61" t="n">
+        <v>2174</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Halifax</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>980</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1168</v>
+      </c>
+      <c r="D62" t="n">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Tazewell</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>438</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1681</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2119</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pulaski</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>565</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1456</v>
+      </c>
+      <c r="D64" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Amherst</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>589</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1347</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1936</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>King George</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>683</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1242</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Mecklenburg</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>871</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1049</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Smyth</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>358</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1529</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1887</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Staunton (City)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C69" t="n">
+        <v>690</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Salem (City)</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>667</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1160</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Wythe</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>394</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1390</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Winchester (City)</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1067</v>
+      </c>
+      <c r="C72" t="n">
+        <v>716</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Carroll</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>360</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1363</v>
+      </c>
+      <c r="D73" t="n">
+        <v>1723</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Hopewell (City)</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1071</v>
+      </c>
+      <c r="C74" t="n">
+        <v>583</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1654</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Greene</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>565</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D75" t="n">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Falls Church (City)</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1355</v>
+      </c>
+      <c r="C76" t="n">
+        <v>205</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Williamsburg (City)</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1327</v>
+      </c>
+      <c r="C77" t="n">
+        <v>201</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Waynesboro (City)</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>714</v>
+      </c>
+      <c r="C78" t="n">
+        <v>805</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1519</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Rockbridge</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>467</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1029</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Russell</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>408</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1086</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1494</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>324</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1149</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>King William</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>419</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1049</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Prince Edward</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>742</v>
+      </c>
+      <c r="C83" t="n">
+        <v>545</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Lee</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>200</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1069</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Giles</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>327</v>
+      </c>
+      <c r="C85" t="n">
+        <v>897</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Nelson</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>512</v>
+      </c>
+      <c r="C86" t="n">
+        <v>711</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Buchanan</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>338</v>
+      </c>
+      <c r="C87" t="n">
+        <v>870</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>500</v>
+      </c>
+      <c r="C88" t="n">
+        <v>707</v>
+      </c>
+      <c r="D88" t="n">
+        <v>1207</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Westmoreland</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>524</v>
+      </c>
+      <c r="C89" t="n">
+        <v>668</v>
+      </c>
+      <c r="D89" t="n">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Covington (City)</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>411</v>
+      </c>
+      <c r="C90" t="n">
+        <v>762</v>
+      </c>
+      <c r="D90" t="n">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Colonial Heights (City)</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>435</v>
+      </c>
+      <c r="C91" t="n">
+        <v>733</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Floyd</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>362</v>
+      </c>
+      <c r="C92" t="n">
+        <v>795</v>
+      </c>
+      <c r="D92" t="n">
+        <v>1157</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Scott</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>173</v>
+      </c>
+      <c r="C93" t="n">
+        <v>956</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Clarke</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>450</v>
+      </c>
+      <c r="C94" t="n">
+        <v>668</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Manassas Park (City)</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>788</v>
+      </c>
+      <c r="C95" t="n">
+        <v>284</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Appomattox</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>281</v>
+      </c>
+      <c r="C96" t="n">
+        <v>778</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Madison</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>336</v>
+      </c>
+      <c r="C97" t="n">
+        <v>715</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Radford (City)</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>565</v>
+      </c>
+      <c r="C98" t="n">
+        <v>483</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Brunswick</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>683</v>
+      </c>
+      <c r="C99" t="n">
+        <v>337</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Bristol (City)</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>286</v>
+      </c>
+      <c r="C100" t="n">
+        <v>727</v>
+      </c>
+      <c r="D100" t="n">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Alleghany</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>290</v>
+      </c>
+      <c r="C101" t="n">
+        <v>691</v>
+      </c>
+      <c r="D101" t="n">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Northampton</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>562</v>
+      </c>
+      <c r="C102" t="n">
+        <v>417</v>
+      </c>
+      <c r="D102" t="n">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Northumberland</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>379</v>
+      </c>
+      <c r="C103" t="n">
+        <v>597</v>
+      </c>
+      <c r="D103" t="n">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Poquoson (City)</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>206</v>
+      </c>
+      <c r="C104" t="n">
+        <v>762</v>
+      </c>
+      <c r="D104" t="n">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Buckingham</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>396</v>
+      </c>
+      <c r="C105" t="n">
+        <v>544</v>
+      </c>
+      <c r="D105" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Patrick</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>233</v>
+      </c>
+      <c r="C106" t="n">
+        <v>700</v>
+      </c>
+      <c r="D106" t="n">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Nottoway</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>444</v>
+      </c>
+      <c r="C107" t="n">
+        <v>489</v>
+      </c>
+      <c r="D107" t="n">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Amelia</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>294</v>
+      </c>
+      <c r="C108" t="n">
+        <v>637</v>
+      </c>
+      <c r="D108" t="n">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Dickenson</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>280</v>
+      </c>
+      <c r="C109" t="n">
+        <v>649</v>
+      </c>
+      <c r="D109" t="n">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Martinsville (City)</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>657</v>
+      </c>
+      <c r="C110" t="n">
+        <v>266</v>
+      </c>
+      <c r="D110" t="n">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Essex</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>475</v>
+      </c>
+      <c r="C111" t="n">
+        <v>371</v>
+      </c>
+      <c r="D111" t="n">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Middlesex</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>271</v>
+      </c>
+      <c r="C112" t="n">
+        <v>540</v>
+      </c>
+      <c r="D112" t="n">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>404</v>
+      </c>
+      <c r="C113" t="n">
+        <v>375</v>
+      </c>
+      <c r="D113" t="n">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Charles City</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>502</v>
+      </c>
+      <c r="C114" t="n">
+        <v>263</v>
+      </c>
+      <c r="D114" t="n">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Grayson</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>172</v>
+      </c>
+      <c r="C115" t="n">
+        <v>576</v>
+      </c>
+      <c r="D115" t="n">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Cumberland</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>302</v>
+      </c>
+      <c r="C116" t="n">
+        <v>420</v>
+      </c>
+      <c r="D116" t="n">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>257</v>
+      </c>
+      <c r="C117" t="n">
+        <v>463</v>
+      </c>
+      <c r="D117" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Lunenburg</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>252</v>
+      </c>
+      <c r="C118" t="n">
+        <v>407</v>
+      </c>
+      <c r="D118" t="n">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Mathews</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>174</v>
+      </c>
+      <c r="C119" t="n">
+        <v>449</v>
+      </c>
+      <c r="D119" t="n">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Franklin (City)</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>408</v>
+      </c>
+      <c r="C120" t="n">
+        <v>185</v>
+      </c>
+      <c r="D120" t="n">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Rappahannock</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>202</v>
+      </c>
+      <c r="C121" t="n">
+        <v>370</v>
+      </c>
+      <c r="D121" t="n">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Greensville</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>390</v>
+      </c>
+      <c r="C122" t="n">
+        <v>166</v>
+      </c>
+      <c r="D122" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Surry</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>289</v>
+      </c>
+      <c r="C123" t="n">
+        <v>252</v>
+      </c>
+      <c r="D123" t="n">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Buena Vista (City)</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>121</v>
+      </c>
+      <c r="C124" t="n">
+        <v>393</v>
+      </c>
+      <c r="D124" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>King and Queen</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>204</v>
+      </c>
+      <c r="C125" t="n">
+        <v>302</v>
+      </c>
+      <c r="D125" t="n">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>169</v>
+      </c>
+      <c r="C126" t="n">
+        <v>307</v>
+      </c>
+      <c r="D126" t="n">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Lexington (City)</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>325</v>
+      </c>
+      <c r="C127" t="n">
+        <v>117</v>
+      </c>
+      <c r="D127" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Galax (City)</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>75</v>
+      </c>
+      <c r="C128" t="n">
+        <v>275</v>
+      </c>
+      <c r="D128" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Bland</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>68</v>
+      </c>
+      <c r="C129" t="n">
+        <v>281</v>
+      </c>
+      <c r="D129" t="n">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Emporia (City)</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>283</v>
+      </c>
+      <c r="C130" t="n">
+        <v>63</v>
+      </c>
+      <c r="D130" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Craig</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>64</v>
+      </c>
+      <c r="C131" t="n">
+        <v>268</v>
+      </c>
+      <c r="D131" t="n">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>77</v>
+      </c>
+      <c r="C132" t="n">
+        <v>243</v>
+      </c>
+      <c r="D132" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Norton (City)</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>71</v>
+      </c>
+      <c r="C133" t="n">
+        <v>227</v>
+      </c>
+      <c r="D133" t="n">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Highland</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>67</v>
+      </c>
+      <c r="C134" t="n">
+        <v>111</v>
+      </c>
+      <c r="D134" t="n">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -4982,77 +6791,349 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>age_band</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>party_bucket</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>ref_voters</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>surge</t>
+          <t>g25</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>surge_pct</t>
+          <t>dropped</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Dem</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1633612</v>
-      </c>
       <c r="C2" t="n">
-        <v>159461</v>
+        <v>135237</v>
       </c>
       <c r="D2" t="n">
-        <v>9.800000000000001</v>
+        <v>60341</v>
+      </c>
+      <c r="E2" t="n">
+        <v>44.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Rep</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>1409220</v>
-      </c>
       <c r="C3" t="n">
-        <v>165921</v>
+        <v>74584</v>
       </c>
       <c r="D3" t="n">
-        <v>11.8</v>
+        <v>27622</v>
+      </c>
+      <c r="E3" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>247938</v>
+      </c>
+      <c r="D4" t="n">
+        <v>84927</v>
+      </c>
+      <c r="E4" t="n">
+        <v>34.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>131390</v>
+      </c>
+      <c r="D5" t="n">
+        <v>38322</v>
+      </c>
+      <c r="E5" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>309929</v>
+      </c>
+      <c r="D6" t="n">
+        <v>79336</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>191191</v>
+      </c>
+      <c r="D7" t="n">
+        <v>43347</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>312125</v>
+      </c>
+      <c r="D8" t="n">
+        <v>69044</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>232185</v>
+      </c>
+      <c r="D9" t="n">
+        <v>42764</v>
+      </c>
+      <c r="E9" t="n">
+        <v>18.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>334848</v>
+      </c>
+      <c r="D10" t="n">
+        <v>57441</v>
+      </c>
+      <c r="E10" t="n">
+        <v>17.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>325743</v>
+      </c>
+      <c r="D11" t="n">
+        <v>43781</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>323224</v>
+      </c>
+      <c r="D12" t="n">
+        <v>39898</v>
+      </c>
+      <c r="E12" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>308856</v>
+      </c>
+      <c r="D13" t="n">
+        <v>30497</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>234700</v>
+      </c>
+      <c r="D14" t="n">
+        <v>32865</v>
+      </c>
+      <c r="E14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>235415</v>
+      </c>
+      <c r="D15" t="n">
+        <v>29732</v>
+      </c>
+      <c r="E15" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>33586</v>
-      </c>
-      <c r="C4" t="n">
-        <v>7033</v>
-      </c>
-      <c r="D4" t="n">
-        <v>20.9</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dem</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5066,13 +7147,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>age_band</t>
+          <t>party_bucket</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -5094,129 +7175,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18-24</t>
+          <t>Dem</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166643</v>
+        <v>1633612</v>
       </c>
       <c r="C2" t="n">
-        <v>41431</v>
+        <v>159461</v>
       </c>
       <c r="D2" t="n">
-        <v>24.9</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25-34</t>
+          <t>Rep</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315837</v>
+        <v>1409220</v>
       </c>
       <c r="C3" t="n">
-        <v>55305</v>
+        <v>165921</v>
       </c>
       <c r="D3" t="n">
-        <v>17.5</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>35-44</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>441836</v>
+        <v>33586</v>
       </c>
       <c r="C4" t="n">
-        <v>59118</v>
+        <v>7033</v>
       </c>
       <c r="D4" t="n">
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>45-54</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>490247</v>
-      </c>
-      <c r="C5" t="n">
-        <v>53832</v>
-      </c>
-      <c r="D5" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>55-64</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>618722</v>
-      </c>
-      <c r="C6" t="n">
-        <v>54902</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>65-74</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>605380</v>
-      </c>
-      <c r="C7" t="n">
-        <v>39697</v>
-      </c>
-      <c r="D7" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>75+</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>435593</v>
-      </c>
-      <c r="C8" t="n">
-        <v>25972</v>
-      </c>
-      <c r="D8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2160</v>
-      </c>
-      <c r="C9" t="n">
-        <v>2158</v>
-      </c>
-      <c r="D9" t="n">
-        <v>99.90000000000001</v>
+        <v>20.9</v>
       </c>
     </row>
   </sheetData>
@@ -5230,13 +7231,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>age_band</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -5258,33 +7259,129 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>18-24</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1417506</v>
+        <v>166643</v>
       </c>
       <c r="C2" t="n">
-        <v>156623</v>
+        <v>41431</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>24.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>25-34</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1654723</v>
+        <v>315837</v>
       </c>
       <c r="C3" t="n">
-        <v>175213</v>
+        <v>55305</v>
       </c>
       <c r="D3" t="n">
-        <v>10.6</v>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>441836</v>
+      </c>
+      <c r="C4" t="n">
+        <v>59118</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>490247</v>
+      </c>
+      <c r="C5" t="n">
+        <v>53832</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>618722</v>
+      </c>
+      <c r="C6" t="n">
+        <v>54902</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>605380</v>
+      </c>
+      <c r="C7" t="n">
+        <v>39697</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>75+</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>435593</v>
+      </c>
+      <c r="C8" t="n">
+        <v>25972</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2160</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2158</v>
+      </c>
+      <c r="D9" t="n">
+        <v>99.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5298,13 +7395,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -5326,177 +7423,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>357830</v>
+        <v>1417506</v>
       </c>
       <c r="C2" t="n">
-        <v>31212</v>
+        <v>156623</v>
       </c>
       <c r="D2" t="n">
-        <v>8.699999999999999</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>280742</v>
+        <v>1654723</v>
       </c>
       <c r="C3" t="n">
-        <v>30319</v>
+        <v>175213</v>
       </c>
       <c r="D3" t="n">
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>212185</v>
-      </c>
-      <c r="C4" t="n">
-        <v>24970</v>
-      </c>
-      <c r="D4" t="n">
-        <v>11.8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>004</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>265510</v>
-      </c>
-      <c r="C5" t="n">
-        <v>25526</v>
-      </c>
-      <c r="D5" t="n">
-        <v>9.6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>005</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>320603</v>
-      </c>
-      <c r="C6" t="n">
-        <v>34925</v>
-      </c>
-      <c r="D6" t="n">
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>292170</v>
-      </c>
-      <c r="C7" t="n">
-        <v>36486</v>
-      </c>
-      <c r="D7" t="n">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>007</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>269849</v>
-      </c>
-      <c r="C8" t="n">
-        <v>31225</v>
-      </c>
-      <c r="D8" t="n">
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>008</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>252038</v>
-      </c>
-      <c r="C9" t="n">
-        <v>21445</v>
-      </c>
-      <c r="D9" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>009</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>278028</v>
-      </c>
-      <c r="C10" t="n">
-        <v>39063</v>
-      </c>
-      <c r="D10" t="n">
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>010</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>274224</v>
-      </c>
-      <c r="C11" t="n">
-        <v>30476</v>
-      </c>
-      <c r="D11" t="n">
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>011</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>273239</v>
-      </c>
-      <c r="C12" t="n">
-        <v>26768</v>
-      </c>
-      <c r="D12" t="n">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
     </row>
   </sheetData>
@@ -5510,13 +7463,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>locality</t>
+          <t>CD</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -5538,193 +7491,177 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fairfax</t>
+          <t>001</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>383154</v>
+        <v>357830</v>
       </c>
       <c r="C2" t="n">
-        <v>36882</v>
+        <v>31212</v>
       </c>
       <c r="D2" t="n">
-        <v>9.6</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Prince William</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>145697</v>
+        <v>280742</v>
       </c>
       <c r="C3" t="n">
-        <v>17252</v>
+        <v>30319</v>
       </c>
       <c r="D3" t="n">
-        <v>11.8</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Loudoun</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>146585</v>
+        <v>212185</v>
       </c>
       <c r="C4" t="n">
-        <v>16674</v>
+        <v>24970</v>
       </c>
       <c r="D4" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Virginia Beach (City)</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150106</v>
+        <v>265510</v>
       </c>
       <c r="C5" t="n">
-        <v>16205</v>
+        <v>25526</v>
       </c>
       <c r="D5" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chesterfield</t>
+          <t>005</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150578</v>
+        <v>320603</v>
       </c>
       <c r="C6" t="n">
-        <v>13353</v>
+        <v>34925</v>
       </c>
       <c r="D6" t="n">
-        <v>8.9</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Henrico</t>
+          <t>006</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>128979</v>
+        <v>292170</v>
       </c>
       <c r="C7" t="n">
-        <v>10635</v>
+        <v>36486</v>
       </c>
       <c r="D7" t="n">
-        <v>8.199999999999999</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chesapeake (City)</t>
+          <t>007</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>86216</v>
+        <v>269849</v>
       </c>
       <c r="C8" t="n">
-        <v>9613</v>
+        <v>31225</v>
       </c>
       <c r="D8" t="n">
-        <v>11.1</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>008</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>83257</v>
+        <v>252038</v>
       </c>
       <c r="C9" t="n">
-        <v>6762</v>
+        <v>21445</v>
       </c>
       <c r="D9" t="n">
-        <v>8.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Norfolk (City)</t>
+          <t>009</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55646</v>
+        <v>278028</v>
       </c>
       <c r="C10" t="n">
-        <v>6573</v>
+        <v>39063</v>
       </c>
       <c r="D10" t="n">
-        <v>11.8</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Richmond (City)</t>
+          <t>010</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>74859</v>
+        <v>274224</v>
       </c>
       <c r="C11" t="n">
-        <v>6322</v>
+        <v>30476</v>
       </c>
       <c r="D11" t="n">
-        <v>8.4</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Spotsylvania</t>
+          <t>011</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>54521</v>
+        <v>273239</v>
       </c>
       <c r="C12" t="n">
-        <v>6304</v>
+        <v>26768</v>
       </c>
       <c r="D12" t="n">
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Newport News (City)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>50574</v>
-      </c>
-      <c r="C13" t="n">
-        <v>6265</v>
-      </c>
-      <c r="D13" t="n">
-        <v>12.4</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5733,6 +7670,234 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>locality</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ref_voters</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>surge</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>surge_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fairfax</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>383154</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36882</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Prince William</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>145697</v>
+      </c>
+      <c r="C3" t="n">
+        <v>17252</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Loudoun</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>146585</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16674</v>
+      </c>
+      <c r="D4" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Virginia Beach (City)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>150106</v>
+      </c>
+      <c r="C5" t="n">
+        <v>16205</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>150578</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13353</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Henrico</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>128979</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10635</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chesapeake (City)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>86216</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9613</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Arlington</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>83257</v>
+      </c>
+      <c r="C9" t="n">
+        <v>6762</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Norfolk (City)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>55646</v>
+      </c>
+      <c r="C10" t="n">
+        <v>6573</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Richmond (City)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>74859</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6322</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spotsylvania</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>54521</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6304</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Newport News (City)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>50574</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6265</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Refresh analysis on new VAN image (Dem_Support_26 score)
- Switch party score Clarity_DemSupport_26 -> Dem_Support_26 (new column);
  rebuild LTV2026_Ref_Base, Dropoff_2025G_Base, Surge_2026_Base (REBUILD=1)
- No-VAN-match referendum voters: 25,494 -> 103 (new registrations now scored)
- Surge 332,415 -> 357,726 (11.5%); drop-off 690,881 -> 682,378 (19.9%);
  net change ~ -324,652; party turnout Rep 52.9% / Dem 45.0%, Dem 53.4% of voters
- Update exec summary, both briefs (PDF/PNG, still 1 page), index, README,
  inventory; generated date -> 2026-05-22

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/LTV2026_Ref_Analysis.xlsx
+++ b/analysis/LTV2026_Ref_Analysis.xlsx
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28208</v>
+        <v>28172</v>
       </c>
     </row>
     <row r="3">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9262</v>
+        <v>9213</v>
       </c>
     </row>
     <row r="4">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7453</v>
+        <v>7417</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5013</v>
+        <v>4975</v>
       </c>
     </row>
     <row r="6">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4859</v>
+        <v>4797</v>
       </c>
     </row>
     <row r="7">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3927</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="8">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1971</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="9">
@@ -931,7 +931,7 @@
         <v>52.2</v>
       </c>
       <c r="E6" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7">
@@ -988,7 +988,7 @@
         <v>58.2</v>
       </c>
       <c r="E9" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="10">
@@ -1086,7 +1086,7 @@
         <v>50.2</v>
       </c>
       <c r="E2" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3">
@@ -1308,16 +1308,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1633612</v>
+        <v>1657450</v>
       </c>
       <c r="C2" t="n">
-        <v>3622724</v>
+        <v>3684105</v>
       </c>
       <c r="D2" t="n">
-        <v>45.1</v>
+        <v>45</v>
       </c>
       <c r="E2" t="n">
-        <v>52.7</v>
+        <v>53.4</v>
       </c>
     </row>
     <row r="3">
@@ -1327,16 +1327,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1409220</v>
+        <v>1444346</v>
       </c>
       <c r="C3" t="n">
-        <v>2659242</v>
+        <v>2728191</v>
       </c>
       <c r="D3" t="n">
-        <v>53</v>
+        <v>52.9</v>
       </c>
       <c r="E3" t="n">
-        <v>45.4</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="4">
@@ -1346,16 +1346,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>59080</v>
+        <v>116</v>
       </c>
       <c r="C4" t="n">
-        <v>104410</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>56.6</v>
+        <v>725</v>
       </c>
       <c r="E4" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3839,7 +3839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3871,10 +3871,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1898003</v>
+        <v>1906755</v>
       </c>
       <c r="C2" t="n">
-        <v>423852</v>
+        <v>424409</v>
       </c>
       <c r="D2" t="n">
         <v>22.3</v>
@@ -3887,29 +3887,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1499364</v>
+        <v>1519706</v>
       </c>
       <c r="C3" t="n">
-        <v>256065</v>
+        <v>257969</v>
       </c>
       <c r="D3" t="n">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>37517</v>
-      </c>
-      <c r="C4" t="n">
-        <v>10964</v>
-      </c>
-      <c r="D4" t="n">
-        <v>29.2</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -3955,10 +3939,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>215728</v>
+        <v>208637</v>
       </c>
       <c r="C2" t="n">
-        <v>90516</v>
+        <v>87710</v>
       </c>
       <c r="D2" t="n">
         <v>42</v>
@@ -3971,13 +3955,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>386335</v>
+        <v>384234</v>
       </c>
       <c r="C3" t="n">
-        <v>125803</v>
+        <v>125706</v>
       </c>
       <c r="D3" t="n">
-        <v>32.6</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="4">
@@ -3987,10 +3971,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>507302</v>
+        <v>505280</v>
       </c>
       <c r="C4" t="n">
-        <v>124584</v>
+        <v>124465</v>
       </c>
       <c r="D4" t="n">
         <v>24.6</v>
@@ -4003,10 +3987,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>549620</v>
+        <v>547394</v>
       </c>
       <c r="C5" t="n">
-        <v>113205</v>
+        <v>112808</v>
       </c>
       <c r="D5" t="n">
         <v>20.6</v>
@@ -4019,13 +4003,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>666243</v>
+        <v>664346</v>
       </c>
       <c r="C6" t="n">
-        <v>102423</v>
+        <v>101967</v>
       </c>
       <c r="D6" t="n">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="7">
@@ -4035,13 +4019,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>636905</v>
+        <v>638302</v>
       </c>
       <c r="C7" t="n">
-        <v>71222</v>
+        <v>70058</v>
       </c>
       <c r="D7" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -4051,13 +4035,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>472749</v>
+        <v>478267</v>
       </c>
       <c r="C8" t="n">
-        <v>63128</v>
+        <v>59664</v>
       </c>
       <c r="D8" t="n">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="9">
@@ -4067,7 +4051,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -4119,13 +4103,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1563439</v>
+        <v>1558834</v>
       </c>
       <c r="C2" t="n">
-        <v>302556</v>
+        <v>297910</v>
       </c>
       <c r="D2" t="n">
-        <v>19.4</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="3">
@@ -4135,13 +4119,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1865930</v>
+        <v>1862184</v>
       </c>
       <c r="C3" t="n">
-        <v>386420</v>
+        <v>382591</v>
       </c>
       <c r="D3" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
     </row>
   </sheetData>
@@ -4187,13 +4171,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>396961</v>
+        <v>396228</v>
       </c>
       <c r="C2" t="n">
-        <v>70343</v>
+        <v>69469</v>
       </c>
       <c r="D2" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="3">
@@ -4203,13 +4187,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>312810</v>
+        <v>311946</v>
       </c>
       <c r="C3" t="n">
-        <v>62387</v>
+        <v>61597</v>
       </c>
       <c r="D3" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="4">
@@ -4219,13 +4203,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>239973</v>
+        <v>239107</v>
       </c>
       <c r="C4" t="n">
-        <v>52758</v>
+        <v>51960</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="5">
@@ -4235,13 +4219,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>307459</v>
+        <v>306713</v>
       </c>
       <c r="C5" t="n">
-        <v>67475</v>
+        <v>66709</v>
       </c>
       <c r="D5" t="n">
-        <v>21.9</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="6">
@@ -4251,13 +4235,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>345424</v>
+        <v>345044</v>
       </c>
       <c r="C6" t="n">
-        <v>59746</v>
+        <v>58803</v>
       </c>
       <c r="D6" t="n">
-        <v>17.3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -4267,13 +4251,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>309206</v>
+        <v>308674</v>
       </c>
       <c r="C7" t="n">
-        <v>53522</v>
+        <v>52728</v>
       </c>
       <c r="D7" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="8">
@@ -4283,13 +4267,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>302051</v>
+        <v>301386</v>
       </c>
       <c r="C8" t="n">
-        <v>63427</v>
+        <v>62801</v>
       </c>
       <c r="D8" t="n">
-        <v>21</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="9">
@@ -4299,13 +4283,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>300435</v>
+        <v>299251</v>
       </c>
       <c r="C9" t="n">
-        <v>69842</v>
+        <v>69103</v>
       </c>
       <c r="D9" t="n">
-        <v>23.2</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="10">
@@ -4315,13 +4299,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>290769</v>
+        <v>290026</v>
       </c>
       <c r="C10" t="n">
-        <v>51804</v>
+        <v>50919</v>
       </c>
       <c r="D10" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="11">
@@ -4331,13 +4315,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>311842</v>
+        <v>310993</v>
       </c>
       <c r="C11" t="n">
-        <v>68094</v>
+        <v>67486</v>
       </c>
       <c r="D11" t="n">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="12">
@@ -4347,13 +4331,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>317954</v>
+        <v>317093</v>
       </c>
       <c r="C12" t="n">
-        <v>71483</v>
+        <v>70803</v>
       </c>
       <c r="D12" t="n">
-        <v>22.5</v>
+        <v>22.3</v>
       </c>
     </row>
   </sheetData>
@@ -4399,13 +4383,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>447400</v>
+        <v>446083</v>
       </c>
       <c r="C2" t="n">
-        <v>101128</v>
+        <v>100138</v>
       </c>
       <c r="D2" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="3">
@@ -4415,13 +4399,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>169052</v>
+        <v>168650</v>
       </c>
       <c r="C3" t="n">
-        <v>39141</v>
+        <v>38862</v>
       </c>
       <c r="D3" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -4431,13 +4415,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>166160</v>
+        <v>165513</v>
       </c>
       <c r="C4" t="n">
-        <v>37715</v>
+        <v>37313</v>
       </c>
       <c r="D4" t="n">
-        <v>22.7</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="5">
@@ -4447,13 +4431,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>170015</v>
+        <v>169391</v>
       </c>
       <c r="C5" t="n">
-        <v>36114</v>
+        <v>35630</v>
       </c>
       <c r="D5" t="n">
-        <v>21.2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -4463,13 +4447,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>170654</v>
+        <v>170422</v>
       </c>
       <c r="C6" t="n">
-        <v>33429</v>
+        <v>33114</v>
       </c>
       <c r="D6" t="n">
-        <v>19.6</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="7">
@@ -4479,13 +4463,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148965</v>
+        <v>148487</v>
       </c>
       <c r="C7" t="n">
-        <v>30621</v>
+        <v>30238</v>
       </c>
       <c r="D7" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="8">
@@ -4495,13 +4479,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99732</v>
+        <v>99223</v>
       </c>
       <c r="C8" t="n">
-        <v>23237</v>
+        <v>22954</v>
       </c>
       <c r="D8" t="n">
-        <v>23.3</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="9">
@@ -4511,13 +4495,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>90278</v>
+        <v>90011</v>
       </c>
       <c r="C9" t="n">
-        <v>21741</v>
+        <v>21517</v>
       </c>
       <c r="D9" t="n">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="10">
@@ -4527,13 +4511,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>96441</v>
+        <v>96216</v>
       </c>
       <c r="C10" t="n">
-        <v>19838</v>
+        <v>19609</v>
       </c>
       <c r="D10" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="11">
@@ -4543,13 +4527,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>62937</v>
+        <v>62719</v>
       </c>
       <c r="C11" t="n">
-        <v>14991</v>
+        <v>14852</v>
       </c>
       <c r="D11" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="12">
@@ -4559,13 +4543,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63595</v>
+        <v>63393</v>
       </c>
       <c r="C12" t="n">
-        <v>14522</v>
+        <v>14321</v>
       </c>
       <c r="D12" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="13">
@@ -4575,13 +4559,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63319</v>
+        <v>63115</v>
       </c>
       <c r="C13" t="n">
-        <v>13274</v>
+        <v>13138</v>
       </c>
       <c r="D13" t="n">
-        <v>21</v>
+        <v>20.8</v>
       </c>
     </row>
   </sheetData>
@@ -4613,31 +4597,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Dem</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26740</v>
+        <v>36174</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dem</t>
+          <t>Rep</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22082</v>
+        <v>28315</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16072</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -4683,13 +4667,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13087</v>
+        <v>13140</v>
       </c>
       <c r="C2" t="n">
-        <v>3702</v>
+        <v>3634</v>
       </c>
       <c r="D2" t="n">
-        <v>28.3</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="3">
@@ -4699,13 +4683,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6662</v>
+        <v>6646</v>
       </c>
       <c r="C3" t="n">
-        <v>1674</v>
+        <v>1659</v>
       </c>
       <c r="D3" t="n">
-        <v>25.1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -4715,45 +4699,45 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10562</v>
+        <v>10559</v>
       </c>
       <c r="C4" t="n">
-        <v>2637</v>
+        <v>2625</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Charlottesville (City)</t>
+          <t>Richmond (City)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18516</v>
+        <v>90011</v>
       </c>
       <c r="C5" t="n">
-        <v>4464</v>
+        <v>21517</v>
       </c>
       <c r="D5" t="n">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Richmond (City)</t>
+          <t>Charlottesville (City)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>90278</v>
+        <v>18646</v>
       </c>
       <c r="C6" t="n">
-        <v>21741</v>
+        <v>4428</v>
       </c>
       <c r="D6" t="n">
-        <v>24.1</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="7">
@@ -4763,61 +4747,61 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10009</v>
+        <v>9956</v>
       </c>
       <c r="C7" t="n">
-        <v>2408</v>
+        <v>2363</v>
       </c>
       <c r="D7" t="n">
-        <v>24.1</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Williamsburg (City)</t>
+          <t>Alexandria (City)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6478</v>
+        <v>62719</v>
       </c>
       <c r="C8" t="n">
-        <v>1544</v>
+        <v>14852</v>
       </c>
       <c r="D8" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Alexandria (City)</t>
+          <t>Buchanan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>62937</v>
+        <v>5406</v>
       </c>
       <c r="C9" t="n">
-        <v>14991</v>
+        <v>1275</v>
       </c>
       <c r="D9" t="n">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Buchanan</t>
+          <t>Williamsburg (City)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5423</v>
+        <v>6572</v>
       </c>
       <c r="C10" t="n">
-        <v>1291</v>
+        <v>1537</v>
       </c>
       <c r="D10" t="n">
-        <v>23.8</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="11">
@@ -4827,13 +4811,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>99732</v>
+        <v>99223</v>
       </c>
       <c r="C11" t="n">
-        <v>23237</v>
+        <v>22954</v>
       </c>
       <c r="D11" t="n">
-        <v>23.3</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="12">
@@ -4843,13 +4827,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>169052</v>
+        <v>168650</v>
       </c>
       <c r="C12" t="n">
-        <v>39141</v>
+        <v>38862</v>
       </c>
       <c r="D12" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -4859,13 +4843,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11092</v>
+        <v>11056</v>
       </c>
       <c r="C13" t="n">
-        <v>2545</v>
+        <v>2510</v>
       </c>
       <c r="D13" t="n">
-        <v>22.9</v>
+        <v>22.7</v>
       </c>
     </row>
   </sheetData>
@@ -4911,13 +4895,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80994</v>
+        <v>81345</v>
       </c>
       <c r="C2" t="n">
-        <v>18911</v>
+        <v>18793</v>
       </c>
       <c r="D2" t="n">
-        <v>99905</v>
+        <v>100138</v>
       </c>
     </row>
     <row r="3">
@@ -4927,13 +4911,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25684</v>
+        <v>25817</v>
       </c>
       <c r="C3" t="n">
-        <v>12959</v>
+        <v>13045</v>
       </c>
       <c r="D3" t="n">
-        <v>38643</v>
+        <v>38862</v>
       </c>
     </row>
     <row r="4">
@@ -4943,13 +4927,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26782</v>
+        <v>26763</v>
       </c>
       <c r="C4" t="n">
-        <v>10591</v>
+        <v>10550</v>
       </c>
       <c r="D4" t="n">
-        <v>37373</v>
+        <v>37313</v>
       </c>
     </row>
     <row r="5">
@@ -4959,13 +4943,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19919</v>
+        <v>19901</v>
       </c>
       <c r="C5" t="n">
-        <v>15660</v>
+        <v>15729</v>
       </c>
       <c r="D5" t="n">
-        <v>35579</v>
+        <v>35630</v>
       </c>
     </row>
     <row r="6">
@@ -4975,13 +4959,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20565</v>
+        <v>20615</v>
       </c>
       <c r="C6" t="n">
-        <v>12467</v>
+        <v>12499</v>
       </c>
       <c r="D6" t="n">
-        <v>33032</v>
+        <v>33114</v>
       </c>
     </row>
     <row r="7">
@@ -4991,13 +4975,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22273</v>
+        <v>22285</v>
       </c>
       <c r="C7" t="n">
-        <v>7984</v>
+        <v>7953</v>
       </c>
       <c r="D7" t="n">
-        <v>30257</v>
+        <v>30238</v>
       </c>
     </row>
     <row r="8">
@@ -5007,13 +4991,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20290</v>
+        <v>20390</v>
       </c>
       <c r="C8" t="n">
-        <v>2580</v>
+        <v>2564</v>
       </c>
       <c r="D8" t="n">
-        <v>22870</v>
+        <v>22954</v>
       </c>
     </row>
     <row r="9">
@@ -5023,13 +5007,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19326</v>
+        <v>19507</v>
       </c>
       <c r="C9" t="n">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="D9" t="n">
-        <v>21335</v>
+        <v>21517</v>
       </c>
     </row>
     <row r="10">
@@ -5039,13 +5023,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10973</v>
+        <v>10984</v>
       </c>
       <c r="C10" t="n">
-        <v>8549</v>
+        <v>8625</v>
       </c>
       <c r="D10" t="n">
-        <v>19522</v>
+        <v>19609</v>
       </c>
     </row>
     <row r="11">
@@ -5055,13 +5039,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12980</v>
+        <v>13130</v>
       </c>
       <c r="C11" t="n">
-        <v>1740</v>
+        <v>1722</v>
       </c>
       <c r="D11" t="n">
-        <v>14720</v>
+        <v>14852</v>
       </c>
     </row>
     <row r="12">
@@ -5071,13 +5055,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11977</v>
+        <v>11993</v>
       </c>
       <c r="C12" t="n">
-        <v>2329</v>
+        <v>2328</v>
       </c>
       <c r="D12" t="n">
-        <v>14306</v>
+        <v>14321</v>
       </c>
     </row>
     <row r="13">
@@ -5087,13 +5071,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7353</v>
+        <v>7375</v>
       </c>
       <c r="C13" t="n">
-        <v>5739</v>
+        <v>5763</v>
       </c>
       <c r="D13" t="n">
-        <v>13092</v>
+        <v>13138</v>
       </c>
     </row>
     <row r="14">
@@ -5103,13 +5087,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9199</v>
+        <v>9179</v>
       </c>
       <c r="C14" t="n">
-        <v>2831</v>
+        <v>2827</v>
       </c>
       <c r="D14" t="n">
-        <v>12030</v>
+        <v>12006</v>
       </c>
     </row>
     <row r="15">
@@ -5119,13 +5103,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5611</v>
+        <v>5634</v>
       </c>
       <c r="C15" t="n">
-        <v>5923</v>
+        <v>6017</v>
       </c>
       <c r="D15" t="n">
-        <v>11534</v>
+        <v>11651</v>
       </c>
     </row>
     <row r="16">
@@ -5135,13 +5119,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7857</v>
+        <v>7866</v>
       </c>
       <c r="C16" t="n">
-        <v>2410</v>
+        <v>2399</v>
       </c>
       <c r="D16" t="n">
-        <v>10267</v>
+        <v>10265</v>
       </c>
     </row>
     <row r="17">
@@ -5151,13 +5135,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7909</v>
+        <v>7907</v>
       </c>
       <c r="C17" t="n">
-        <v>1648</v>
+        <v>1628</v>
       </c>
       <c r="D17" t="n">
-        <v>9557</v>
+        <v>9535</v>
       </c>
     </row>
     <row r="18">
@@ -5167,13 +5151,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3131</v>
+        <v>3157</v>
       </c>
       <c r="C18" t="n">
-        <v>6129</v>
+        <v>6158</v>
       </c>
       <c r="D18" t="n">
-        <v>9260</v>
+        <v>9315</v>
       </c>
     </row>
     <row r="19">
@@ -5183,13 +5167,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5203</v>
+        <v>5163</v>
       </c>
       <c r="C19" t="n">
-        <v>2909</v>
+        <v>2946</v>
       </c>
       <c r="D19" t="n">
-        <v>8112</v>
+        <v>8109</v>
       </c>
     </row>
     <row r="20">
@@ -5199,13 +5183,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5206</v>
+        <v>5190</v>
       </c>
       <c r="C20" t="n">
-        <v>2730</v>
+        <v>2745</v>
       </c>
       <c r="D20" t="n">
-        <v>7936</v>
+        <v>7935</v>
       </c>
     </row>
     <row r="21">
@@ -5215,13 +5199,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2559</v>
+        <v>2545</v>
       </c>
       <c r="C21" t="n">
-        <v>4559</v>
+        <v>4592</v>
       </c>
       <c r="D21" t="n">
-        <v>7118</v>
+        <v>7137</v>
       </c>
     </row>
     <row r="22">
@@ -5231,13 +5215,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5668</v>
+        <v>5674</v>
       </c>
       <c r="C22" t="n">
-        <v>1405</v>
+        <v>1410</v>
       </c>
       <c r="D22" t="n">
-        <v>7073</v>
+        <v>7084</v>
       </c>
     </row>
     <row r="23">
@@ -5247,45 +5231,45 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3780</v>
+        <v>3730</v>
       </c>
       <c r="C23" t="n">
-        <v>3255</v>
+        <v>3243</v>
       </c>
       <c r="D23" t="n">
-        <v>7035</v>
+        <v>6973</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Roanoke (City)</t>
+          <t>Frederick</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4631</v>
+        <v>2118</v>
       </c>
       <c r="C24" t="n">
-        <v>2044</v>
+        <v>4583</v>
       </c>
       <c r="D24" t="n">
-        <v>6675</v>
+        <v>6701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Frederick</t>
+          <t>Roanoke (City)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2117</v>
+        <v>4618</v>
       </c>
       <c r="C25" t="n">
-        <v>4484</v>
+        <v>2032</v>
       </c>
       <c r="D25" t="n">
-        <v>6601</v>
+        <v>6650</v>
       </c>
     </row>
     <row r="26">
@@ -5295,13 +5279,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2190</v>
+        <v>2179</v>
       </c>
       <c r="C26" t="n">
-        <v>3754</v>
+        <v>3778</v>
       </c>
       <c r="D26" t="n">
-        <v>5944</v>
+        <v>5957</v>
       </c>
     </row>
     <row r="27">
@@ -5311,13 +5295,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2437</v>
+        <v>2401</v>
       </c>
       <c r="C27" t="n">
-        <v>3170</v>
+        <v>3172</v>
       </c>
       <c r="D27" t="n">
-        <v>5607</v>
+        <v>5573</v>
       </c>
     </row>
     <row r="28">
@@ -5327,13 +5311,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1179</v>
+        <v>1172</v>
       </c>
       <c r="C28" t="n">
-        <v>4218</v>
+        <v>4319</v>
       </c>
       <c r="D28" t="n">
-        <v>5397</v>
+        <v>5491</v>
       </c>
     </row>
     <row r="29">
@@ -5343,13 +5327,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2517</v>
+        <v>2531</v>
       </c>
       <c r="C29" t="n">
-        <v>2625</v>
+        <v>2620</v>
       </c>
       <c r="D29" t="n">
-        <v>5142</v>
+        <v>5151</v>
       </c>
     </row>
     <row r="30">
@@ -5359,13 +5343,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1396</v>
+        <v>1388</v>
       </c>
       <c r="C30" t="n">
-        <v>3402</v>
+        <v>3440</v>
       </c>
       <c r="D30" t="n">
-        <v>4798</v>
+        <v>4828</v>
       </c>
     </row>
     <row r="31">
@@ -5375,13 +5359,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="C31" t="n">
-        <v>3563</v>
+        <v>3601</v>
       </c>
       <c r="D31" t="n">
-        <v>4596</v>
+        <v>4633</v>
       </c>
     </row>
     <row r="32">
@@ -5391,13 +5375,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4037</v>
+        <v>4094</v>
       </c>
       <c r="C32" t="n">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D32" t="n">
-        <v>4373</v>
+        <v>4428</v>
       </c>
     </row>
     <row r="33">
@@ -5407,13 +5391,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1653</v>
+        <v>1657</v>
       </c>
       <c r="C33" t="n">
-        <v>2564</v>
+        <v>2607</v>
       </c>
       <c r="D33" t="n">
-        <v>4217</v>
+        <v>4264</v>
       </c>
     </row>
     <row r="34">
@@ -5423,13 +5407,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="C34" t="n">
-        <v>2943</v>
+        <v>3011</v>
       </c>
       <c r="D34" t="n">
-        <v>3898</v>
+        <v>3964</v>
       </c>
     </row>
     <row r="35">
@@ -5439,13 +5423,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3031</v>
+        <v>3057</v>
       </c>
       <c r="C35" t="n">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D35" t="n">
-        <v>3609</v>
+        <v>3634</v>
       </c>
     </row>
     <row r="36">
@@ -5455,13 +5439,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>781</v>
+        <v>765</v>
       </c>
       <c r="C36" t="n">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="D36" t="n">
-        <v>3521</v>
+        <v>3501</v>
       </c>
     </row>
     <row r="37">
@@ -5471,13 +5455,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1132</v>
+        <v>1121</v>
       </c>
       <c r="C37" t="n">
-        <v>2354</v>
+        <v>2366</v>
       </c>
       <c r="D37" t="n">
-        <v>3486</v>
+        <v>3487</v>
       </c>
     </row>
     <row r="38">
@@ -5487,10 +5471,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>909</v>
+        <v>880</v>
       </c>
       <c r="C38" t="n">
-        <v>2269</v>
+        <v>2298</v>
       </c>
       <c r="D38" t="n">
         <v>3178</v>
@@ -5503,13 +5487,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1090</v>
+        <v>1104</v>
       </c>
       <c r="C39" t="n">
-        <v>1999</v>
+        <v>2042</v>
       </c>
       <c r="D39" t="n">
-        <v>3089</v>
+        <v>3146</v>
       </c>
     </row>
     <row r="40">
@@ -5519,13 +5503,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1173</v>
+        <v>1151</v>
       </c>
       <c r="C40" t="n">
-        <v>1848</v>
+        <v>1852</v>
       </c>
       <c r="D40" t="n">
-        <v>3021</v>
+        <v>3003</v>
       </c>
     </row>
     <row r="41">
@@ -5535,13 +5519,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="C41" t="n">
-        <v>1903</v>
+        <v>1928</v>
       </c>
       <c r="D41" t="n">
-        <v>2970</v>
+        <v>2994</v>
       </c>
     </row>
     <row r="42">
@@ -5551,13 +5535,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="C42" t="n">
-        <v>1791</v>
+        <v>1824</v>
       </c>
       <c r="D42" t="n">
-        <v>2924</v>
+        <v>2951</v>
       </c>
     </row>
     <row r="43">
@@ -5567,13 +5551,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="C43" t="n">
-        <v>1374</v>
+        <v>1417</v>
       </c>
       <c r="D43" t="n">
-        <v>2682</v>
+        <v>2726</v>
       </c>
     </row>
     <row r="44">
@@ -5583,61 +5567,61 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>739</v>
+        <v>725</v>
       </c>
       <c r="C44" t="n">
-        <v>1907</v>
+        <v>1938</v>
       </c>
       <c r="D44" t="n">
-        <v>2646</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Manassas (City)</t>
+          <t>Warren</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1851</v>
+        <v>802</v>
       </c>
       <c r="C45" t="n">
-        <v>780</v>
+        <v>1842</v>
       </c>
       <c r="D45" t="n">
-        <v>2631</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Fredericksburg (City)</t>
+          <t>Manassas (City)</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2065</v>
+        <v>1850</v>
       </c>
       <c r="C46" t="n">
-        <v>545</v>
+        <v>778</v>
       </c>
       <c r="D46" t="n">
-        <v>2610</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Fredericksburg (City)</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>798</v>
+        <v>2081</v>
       </c>
       <c r="C47" t="n">
-        <v>1803</v>
+        <v>544</v>
       </c>
       <c r="D47" t="n">
-        <v>2601</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="48">
@@ -5647,13 +5631,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1451</v>
+        <v>1455</v>
       </c>
       <c r="C48" t="n">
-        <v>1138</v>
+        <v>1158</v>
       </c>
       <c r="D48" t="n">
-        <v>2589</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="49">
@@ -5663,13 +5647,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="C49" t="n">
-        <v>1930</v>
+        <v>1963</v>
       </c>
       <c r="D49" t="n">
-        <v>2587</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="50">
@@ -5679,93 +5663,93 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="C50" t="n">
-        <v>1945</v>
+        <v>1992</v>
       </c>
       <c r="D50" t="n">
-        <v>2546</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Danville (City)</t>
+          <t>Goochland</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1844</v>
+        <v>986</v>
       </c>
       <c r="C51" t="n">
-        <v>690</v>
+        <v>1531</v>
       </c>
       <c r="D51" t="n">
-        <v>2534</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Goochland</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>989</v>
+        <v>491</v>
       </c>
       <c r="C52" t="n">
-        <v>1517</v>
+        <v>2019</v>
       </c>
       <c r="D52" t="n">
-        <v>2506</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>Danville (City)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>497</v>
+        <v>1821</v>
       </c>
       <c r="C53" t="n">
-        <v>1935</v>
+        <v>683</v>
       </c>
       <c r="D53" t="n">
-        <v>2432</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Petersburg (City)</t>
+          <t>Prince George</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2247</v>
+        <v>1056</v>
       </c>
       <c r="C54" t="n">
-        <v>132</v>
+        <v>1336</v>
       </c>
       <c r="D54" t="n">
-        <v>2379</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Prince George</t>
+          <t>Petersburg (City)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1054</v>
+        <v>2234</v>
       </c>
       <c r="C55" t="n">
-        <v>1316</v>
+        <v>129</v>
       </c>
       <c r="D55" t="n">
-        <v>2370</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="56">
@@ -5775,45 +5759,45 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="C56" t="n">
-        <v>1536</v>
+        <v>1546</v>
       </c>
       <c r="D56" t="n">
-        <v>2258</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fairfax (City)</t>
+          <t>Dinwiddie</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1823</v>
+        <v>955</v>
       </c>
       <c r="C57" t="n">
-        <v>420</v>
+        <v>1294</v>
       </c>
       <c r="D57" t="n">
-        <v>2243</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Dinwiddie</t>
+          <t>Fairfax (City)</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>954</v>
+        <v>1833</v>
       </c>
       <c r="C58" t="n">
-        <v>1283</v>
+        <v>411</v>
       </c>
       <c r="D58" t="n">
-        <v>2237</v>
+        <v>2244</v>
       </c>
     </row>
     <row r="59">
@@ -5823,13 +5807,13 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>989</v>
+        <v>965</v>
       </c>
       <c r="C59" t="n">
-        <v>1216</v>
+        <v>1237</v>
       </c>
       <c r="D59" t="n">
-        <v>2205</v>
+        <v>2202</v>
       </c>
     </row>
     <row r="60">
@@ -5839,10 +5823,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="C60" t="n">
-        <v>1660</v>
+        <v>1667</v>
       </c>
       <c r="D60" t="n">
         <v>2197</v>
@@ -5855,45 +5839,45 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>951</v>
+        <v>959</v>
       </c>
       <c r="C61" t="n">
-        <v>1223</v>
+        <v>1238</v>
       </c>
       <c r="D61" t="n">
-        <v>2174</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Tazewell</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>980</v>
+        <v>423</v>
       </c>
       <c r="C62" t="n">
-        <v>1168</v>
+        <v>1718</v>
       </c>
       <c r="D62" t="n">
-        <v>2148</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tazewell</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>438</v>
+        <v>968</v>
       </c>
       <c r="C63" t="n">
-        <v>1681</v>
+        <v>1158</v>
       </c>
       <c r="D63" t="n">
-        <v>2119</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="64">
@@ -5903,13 +5887,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="C64" t="n">
-        <v>1456</v>
+        <v>1471</v>
       </c>
       <c r="D64" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="65">
@@ -5919,13 +5903,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>589</v>
+        <v>577</v>
       </c>
       <c r="C65" t="n">
-        <v>1347</v>
+        <v>1367</v>
       </c>
       <c r="D65" t="n">
-        <v>1936</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="66">
@@ -5935,45 +5919,45 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="C66" t="n">
-        <v>1242</v>
+        <v>1262</v>
       </c>
       <c r="D66" t="n">
-        <v>1925</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mecklenburg</t>
+          <t>Smyth</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>871</v>
+        <v>349</v>
       </c>
       <c r="C67" t="n">
-        <v>1049</v>
+        <v>1574</v>
       </c>
       <c r="D67" t="n">
-        <v>1920</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Smyth</t>
+          <t>Mecklenburg</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>358</v>
+        <v>860</v>
       </c>
       <c r="C68" t="n">
-        <v>1529</v>
+        <v>1041</v>
       </c>
       <c r="D68" t="n">
-        <v>1887</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="69">
@@ -5983,13 +5967,13 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1177</v>
+        <v>1179</v>
       </c>
       <c r="C69" t="n">
-        <v>690</v>
+        <v>699</v>
       </c>
       <c r="D69" t="n">
-        <v>1867</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="70">
@@ -5999,13 +5983,13 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="C70" t="n">
-        <v>1160</v>
+        <v>1153</v>
       </c>
       <c r="D70" t="n">
-        <v>1827</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="71">
@@ -6015,13 +5999,13 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C71" t="n">
-        <v>1390</v>
+        <v>1410</v>
       </c>
       <c r="D71" t="n">
-        <v>1784</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="72">
@@ -6031,13 +6015,13 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="C72" t="n">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="D72" t="n">
-        <v>1783</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="73">
@@ -6047,13 +6031,13 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="C73" t="n">
-        <v>1363</v>
+        <v>1368</v>
       </c>
       <c r="D73" t="n">
-        <v>1723</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="74">
@@ -6063,13 +6047,13 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1071</v>
+        <v>1074</v>
       </c>
       <c r="C74" t="n">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D74" t="n">
-        <v>1654</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="75">
@@ -6079,13 +6063,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C75" t="n">
-        <v>1034</v>
+        <v>1047</v>
       </c>
       <c r="D75" t="n">
-        <v>1599</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="76">
@@ -6095,29 +6079,29 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1355</v>
+        <v>1378</v>
       </c>
       <c r="C76" t="n">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D76" t="n">
-        <v>1560</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Williamsburg (City)</t>
+          <t>Russell</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1327</v>
+        <v>403</v>
       </c>
       <c r="C77" t="n">
-        <v>201</v>
+        <v>1159</v>
       </c>
       <c r="D77" t="n">
-        <v>1528</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="78">
@@ -6127,45 +6111,45 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="C78" t="n">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="D78" t="n">
-        <v>1519</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Rockbridge</t>
+          <t>Williamsburg (City)</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>467</v>
+        <v>1337</v>
       </c>
       <c r="C79" t="n">
-        <v>1029</v>
+        <v>200</v>
       </c>
       <c r="D79" t="n">
-        <v>1496</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Russell</t>
+          <t>Rockbridge</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>408</v>
+        <v>461</v>
       </c>
       <c r="C80" t="n">
-        <v>1086</v>
+        <v>1047</v>
       </c>
       <c r="D80" t="n">
-        <v>1494</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="81">
@@ -6175,13 +6159,13 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C81" t="n">
-        <v>1149</v>
+        <v>1186</v>
       </c>
       <c r="D81" t="n">
-        <v>1473</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="82">
@@ -6191,109 +6175,109 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="C82" t="n">
-        <v>1049</v>
+        <v>1072</v>
       </c>
       <c r="D82" t="n">
-        <v>1468</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Prince Edward</t>
+          <t>Lee</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>742</v>
+        <v>199</v>
       </c>
       <c r="C83" t="n">
-        <v>545</v>
+        <v>1148</v>
       </c>
       <c r="D83" t="n">
-        <v>1287</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Lee</t>
+          <t>Prince Edward</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>200</v>
+        <v>733</v>
       </c>
       <c r="C84" t="n">
-        <v>1069</v>
+        <v>550</v>
       </c>
       <c r="D84" t="n">
-        <v>1269</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Giles</t>
+          <t>Buchanan</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="C85" t="n">
-        <v>897</v>
+        <v>941</v>
       </c>
       <c r="D85" t="n">
-        <v>1224</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Nelson</t>
+          <t>Giles</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>512</v>
+        <v>319</v>
       </c>
       <c r="C86" t="n">
-        <v>711</v>
+        <v>918</v>
       </c>
       <c r="D86" t="n">
-        <v>1223</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Buchanan</t>
+          <t>Southampton</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>338</v>
+        <v>491</v>
       </c>
       <c r="C87" t="n">
-        <v>870</v>
+        <v>720</v>
       </c>
       <c r="D87" t="n">
-        <v>1208</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Southampton</t>
+          <t>Nelson</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C88" t="n">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="D88" t="n">
-        <v>1207</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="89">
@@ -6303,13 +6287,13 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>524</v>
+        <v>514</v>
       </c>
       <c r="C89" t="n">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="D89" t="n">
-        <v>1192</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="90">
@@ -6319,13 +6303,13 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C90" t="n">
-        <v>762</v>
+        <v>779</v>
       </c>
       <c r="D90" t="n">
-        <v>1173</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="91">
@@ -6338,10 +6322,10 @@
         <v>435</v>
       </c>
       <c r="C91" t="n">
-        <v>733</v>
+        <v>743</v>
       </c>
       <c r="D91" t="n">
-        <v>1168</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="92">
@@ -6351,13 +6335,13 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="C92" t="n">
-        <v>795</v>
+        <v>803</v>
       </c>
       <c r="D92" t="n">
-        <v>1157</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="93">
@@ -6367,13 +6351,13 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C93" t="n">
-        <v>956</v>
+        <v>979</v>
       </c>
       <c r="D93" t="n">
-        <v>1129</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="94">
@@ -6383,13 +6367,13 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="C94" t="n">
         <v>668</v>
       </c>
       <c r="D94" t="n">
-        <v>1118</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="95">
@@ -6399,13 +6383,13 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="C95" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D95" t="n">
-        <v>1072</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="96">
@@ -6415,13 +6399,13 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C96" t="n">
-        <v>778</v>
+        <v>792</v>
       </c>
       <c r="D96" t="n">
-        <v>1059</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="97">
@@ -6431,13 +6415,13 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C97" t="n">
-        <v>715</v>
+        <v>724</v>
       </c>
       <c r="D97" t="n">
-        <v>1051</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="98">
@@ -6447,13 +6431,13 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>565</v>
+        <v>554</v>
       </c>
       <c r="C98" t="n">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="D98" t="n">
-        <v>1048</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="99">
@@ -6463,173 +6447,173 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="C99" t="n">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D99" t="n">
-        <v>1020</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Bristol (City)</t>
+          <t>Alleghany</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C100" t="n">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="D100" t="n">
-        <v>1013</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Alleghany</t>
+          <t>Bristol (City)</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="C101" t="n">
-        <v>691</v>
+        <v>719</v>
       </c>
       <c r="D101" t="n">
-        <v>981</v>
+        <v>996</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Northampton</t>
+          <t>Poquoson (City)</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>562</v>
+        <v>210</v>
       </c>
       <c r="C102" t="n">
-        <v>417</v>
+        <v>784</v>
       </c>
       <c r="D102" t="n">
-        <v>979</v>
+        <v>994</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Northumberland</t>
+          <t>Dickenson</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>379</v>
+        <v>274</v>
       </c>
       <c r="C103" t="n">
-        <v>597</v>
+        <v>697</v>
       </c>
       <c r="D103" t="n">
-        <v>976</v>
+        <v>971</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Poquoson (City)</t>
+          <t>Northampton</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>206</v>
+        <v>558</v>
       </c>
       <c r="C104" t="n">
-        <v>762</v>
+        <v>409</v>
       </c>
       <c r="D104" t="n">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Buckingham</t>
+          <t>Northumberland</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>396</v>
+        <v>378</v>
       </c>
       <c r="C105" t="n">
-        <v>544</v>
+        <v>586</v>
       </c>
       <c r="D105" t="n">
-        <v>940</v>
+        <v>964</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Patrick</t>
+          <t>Amelia</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>233</v>
+        <v>294</v>
       </c>
       <c r="C106" t="n">
-        <v>700</v>
+        <v>652</v>
       </c>
       <c r="D106" t="n">
-        <v>933</v>
+        <v>946</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Nottoway</t>
+          <t>Buckingham</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>444</v>
+        <v>396</v>
       </c>
       <c r="C107" t="n">
-        <v>489</v>
+        <v>549</v>
       </c>
       <c r="D107" t="n">
-        <v>933</v>
+        <v>945</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Amelia</t>
+          <t>Patrick</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>294</v>
+        <v>230</v>
       </c>
       <c r="C108" t="n">
-        <v>637</v>
+        <v>703</v>
       </c>
       <c r="D108" t="n">
-        <v>931</v>
+        <v>933</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Dickenson</t>
+          <t>Nottoway</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>280</v>
+        <v>436</v>
       </c>
       <c r="C109" t="n">
-        <v>649</v>
+        <v>490</v>
       </c>
       <c r="D109" t="n">
-        <v>929</v>
+        <v>926</v>
       </c>
     </row>
     <row r="110">
@@ -6639,13 +6623,13 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>657</v>
+        <v>644</v>
       </c>
       <c r="C110" t="n">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="D110" t="n">
-        <v>923</v>
+        <v>914</v>
       </c>
     </row>
     <row r="111">
@@ -6655,13 +6639,13 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C111" t="n">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="D111" t="n">
-        <v>846</v>
+        <v>852</v>
       </c>
     </row>
     <row r="112">
@@ -6671,13 +6655,13 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C112" t="n">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="D112" t="n">
-        <v>811</v>
+        <v>800</v>
       </c>
     </row>
     <row r="113">
@@ -6687,13 +6671,13 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="C113" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D113" t="n">
-        <v>779</v>
+        <v>773</v>
       </c>
     </row>
     <row r="114">
@@ -6703,13 +6687,13 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="C114" t="n">
         <v>263</v>
       </c>
       <c r="D114" t="n">
-        <v>765</v>
+        <v>760</v>
       </c>
     </row>
     <row r="115">
@@ -6719,45 +6703,45 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C115" t="n">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D115" t="n">
-        <v>748</v>
+        <v>743</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Cumberland</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>302</v>
+        <v>251</v>
       </c>
       <c r="C116" t="n">
-        <v>420</v>
+        <v>473</v>
       </c>
       <c r="D116" t="n">
-        <v>722</v>
+        <v>724</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Cumberland</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>257</v>
+        <v>293</v>
       </c>
       <c r="C117" t="n">
-        <v>463</v>
+        <v>418</v>
       </c>
       <c r="D117" t="n">
-        <v>720</v>
+        <v>711</v>
       </c>
     </row>
     <row r="118">
@@ -6767,13 +6751,13 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C118" t="n">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="D118" t="n">
-        <v>659</v>
+        <v>648</v>
       </c>
     </row>
     <row r="119">
@@ -6783,13 +6767,13 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C119" t="n">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D119" t="n">
-        <v>623</v>
+        <v>630</v>
       </c>
     </row>
     <row r="120">
@@ -6799,13 +6783,13 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="C120" t="n">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D120" t="n">
-        <v>593</v>
+        <v>586</v>
       </c>
     </row>
     <row r="121">
@@ -6815,13 +6799,13 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C121" t="n">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="D121" t="n">
-        <v>572</v>
+        <v>580</v>
       </c>
     </row>
     <row r="122">
@@ -6831,13 +6815,13 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="C122" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D122" t="n">
-        <v>556</v>
+        <v>545</v>
       </c>
     </row>
     <row r="123">
@@ -6847,13 +6831,13 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C123" t="n">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="D123" t="n">
-        <v>541</v>
+        <v>528</v>
       </c>
     </row>
     <row r="124">
@@ -6866,10 +6850,10 @@
         <v>121</v>
       </c>
       <c r="C124" t="n">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="D124" t="n">
-        <v>514</v>
+        <v>518</v>
       </c>
     </row>
     <row r="125">
@@ -6879,13 +6863,13 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C125" t="n">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="D125" t="n">
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="126">
@@ -6895,13 +6879,13 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C126" t="n">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D126" t="n">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="127">
@@ -6911,13 +6895,13 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="C127" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D127" t="n">
-        <v>442</v>
+        <v>438</v>
       </c>
     </row>
     <row r="128">
@@ -6927,13 +6911,13 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C128" t="n">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="D128" t="n">
-        <v>350</v>
+        <v>365</v>
       </c>
     </row>
     <row r="129">
@@ -6943,13 +6927,13 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C129" t="n">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="D129" t="n">
-        <v>349</v>
+        <v>359</v>
       </c>
     </row>
     <row r="130">
@@ -6959,13 +6943,13 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C130" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D130" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="131">
@@ -6975,13 +6959,13 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C131" t="n">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D131" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="132">
@@ -6994,10 +6978,10 @@
         <v>77</v>
       </c>
       <c r="C132" t="n">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D132" t="n">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
     <row r="133">
@@ -7007,13 +6991,13 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C133" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D133" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="134">
@@ -7023,13 +7007,13 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C134" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D134" t="n">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -7085,13 +7069,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>135237</v>
+        <v>133494</v>
       </c>
       <c r="D2" t="n">
-        <v>60341</v>
+        <v>59824</v>
       </c>
       <c r="E2" t="n">
-        <v>44.6</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="3">
@@ -7106,13 +7090,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>74584</v>
+        <v>75143</v>
       </c>
       <c r="D3" t="n">
-        <v>27622</v>
+        <v>27886</v>
       </c>
       <c r="E3" t="n">
-        <v>37</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="4">
@@ -7127,13 +7111,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>247938</v>
+        <v>250155</v>
       </c>
       <c r="D4" t="n">
-        <v>84927</v>
+        <v>86361</v>
       </c>
       <c r="E4" t="n">
-        <v>34.3</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="5">
@@ -7148,13 +7132,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>131390</v>
+        <v>134079</v>
       </c>
       <c r="D5" t="n">
-        <v>38322</v>
+        <v>39345</v>
       </c>
       <c r="E5" t="n">
-        <v>29.2</v>
+        <v>29.3</v>
       </c>
     </row>
     <row r="6">
@@ -7169,13 +7153,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>309929</v>
+        <v>310958</v>
       </c>
       <c r="D6" t="n">
-        <v>79336</v>
+        <v>80028</v>
       </c>
       <c r="E6" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="7">
@@ -7190,13 +7174,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>191191</v>
+        <v>194322</v>
       </c>
       <c r="D7" t="n">
-        <v>43347</v>
+        <v>44437</v>
       </c>
       <c r="E7" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="8">
@@ -7211,13 +7195,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>312125</v>
+        <v>313467</v>
       </c>
       <c r="D8" t="n">
-        <v>69044</v>
+        <v>69465</v>
       </c>
       <c r="E8" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="9">
@@ -7232,13 +7216,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>232185</v>
+        <v>233927</v>
       </c>
       <c r="D9" t="n">
-        <v>42764</v>
+        <v>43343</v>
       </c>
       <c r="E9" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="10">
@@ -7253,10 +7237,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>334848</v>
+        <v>335827</v>
       </c>
       <c r="D10" t="n">
-        <v>57441</v>
+        <v>57723</v>
       </c>
       <c r="E10" t="n">
         <v>17.2</v>
@@ -7274,13 +7258,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>325743</v>
+        <v>328519</v>
       </c>
       <c r="D11" t="n">
-        <v>43781</v>
+        <v>44244</v>
       </c>
       <c r="E11" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="12">
@@ -7295,13 +7279,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>323224</v>
+        <v>324460</v>
       </c>
       <c r="D12" t="n">
-        <v>39898</v>
+        <v>39589</v>
       </c>
       <c r="E12" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="13">
@@ -7316,13 +7300,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>308856</v>
+        <v>313842</v>
       </c>
       <c r="D13" t="n">
-        <v>30497</v>
+        <v>30469</v>
       </c>
       <c r="E13" t="n">
-        <v>9.9</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -7337,13 +7321,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>234700</v>
+        <v>238393</v>
       </c>
       <c r="D14" t="n">
-        <v>32865</v>
+        <v>31419</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="15">
@@ -7358,13 +7342,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>235415</v>
+        <v>239874</v>
       </c>
       <c r="D15" t="n">
-        <v>29732</v>
+        <v>28245</v>
       </c>
       <c r="E15" t="n">
-        <v>12.6</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="16">
@@ -7379,7 +7363,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -7431,13 +7415,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1633612</v>
+        <v>1657450</v>
       </c>
       <c r="C2" t="n">
-        <v>159461</v>
+        <v>175104</v>
       </c>
       <c r="D2" t="n">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="3">
@@ -7447,13 +7431,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1409220</v>
+        <v>1444346</v>
       </c>
       <c r="C3" t="n">
-        <v>165921</v>
+        <v>182609</v>
       </c>
       <c r="D3" t="n">
-        <v>11.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="4">
@@ -7463,13 +7447,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33586</v>
+        <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>7033</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>20.9</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -7515,13 +7499,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166643</v>
+        <v>175031</v>
       </c>
       <c r="C2" t="n">
-        <v>41431</v>
+        <v>54104</v>
       </c>
       <c r="D2" t="n">
-        <v>24.9</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="3">
@@ -7531,13 +7515,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315837</v>
+        <v>316406</v>
       </c>
       <c r="C3" t="n">
-        <v>55305</v>
+        <v>57878</v>
       </c>
       <c r="D3" t="n">
-        <v>17.5</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="4">
@@ -7547,13 +7531,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>441836</v>
+        <v>442097</v>
       </c>
       <c r="C4" t="n">
-        <v>59118</v>
+        <v>61282</v>
       </c>
       <c r="D4" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="5">
@@ -7563,13 +7547,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>490247</v>
+        <v>489973</v>
       </c>
       <c r="C5" t="n">
-        <v>53832</v>
+        <v>55387</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="6">
@@ -7579,13 +7563,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>618722</v>
+        <v>619188</v>
       </c>
       <c r="C6" t="n">
-        <v>54902</v>
+        <v>56809</v>
       </c>
       <c r="D6" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -7595,13 +7579,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>605380</v>
+        <v>609813</v>
       </c>
       <c r="C7" t="n">
-        <v>39697</v>
+        <v>41569</v>
       </c>
       <c r="D7" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="8">
@@ -7611,13 +7595,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>435593</v>
+        <v>445911</v>
       </c>
       <c r="C8" t="n">
-        <v>25972</v>
+        <v>27308</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="9">
@@ -7627,13 +7611,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2160</v>
+        <v>3390</v>
       </c>
       <c r="C9" t="n">
-        <v>2158</v>
+        <v>3389</v>
       </c>
       <c r="D9" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -7679,13 +7663,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1417506</v>
+        <v>1429269</v>
       </c>
       <c r="C2" t="n">
-        <v>156623</v>
+        <v>168345</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="3">
@@ -7695,13 +7679,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1654723</v>
+        <v>1668186</v>
       </c>
       <c r="C3" t="n">
-        <v>175213</v>
+        <v>188593</v>
       </c>
       <c r="D3" t="n">
-        <v>10.6</v>
+        <v>11.3</v>
       </c>
     </row>
   </sheetData>
@@ -7747,13 +7731,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>357830</v>
+        <v>361010</v>
       </c>
       <c r="C2" t="n">
-        <v>31212</v>
+        <v>34251</v>
       </c>
       <c r="D2" t="n">
-        <v>8.699999999999999</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="3">
@@ -7763,13 +7747,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>280742</v>
+        <v>282484</v>
       </c>
       <c r="C3" t="n">
-        <v>30319</v>
+        <v>32135</v>
       </c>
       <c r="D3" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="4">
@@ -7779,13 +7763,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>212185</v>
+        <v>213583</v>
       </c>
       <c r="C4" t="n">
-        <v>24970</v>
+        <v>26436</v>
       </c>
       <c r="D4" t="n">
-        <v>11.8</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5">
@@ -7795,13 +7779,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>265510</v>
+        <v>267204</v>
       </c>
       <c r="C5" t="n">
-        <v>25526</v>
+        <v>27200</v>
       </c>
       <c r="D5" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="6">
@@ -7811,13 +7795,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>320603</v>
+        <v>324222</v>
       </c>
       <c r="C6" t="n">
-        <v>34925</v>
+        <v>37981</v>
       </c>
       <c r="D6" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="7">
@@ -7827,13 +7811,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>292170</v>
+        <v>294703</v>
       </c>
       <c r="C7" t="n">
-        <v>36486</v>
+        <v>38757</v>
       </c>
       <c r="D7" t="n">
-        <v>12.5</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="8">
@@ -7843,13 +7827,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>269849</v>
+        <v>271855</v>
       </c>
       <c r="C8" t="n">
-        <v>31225</v>
+        <v>33270</v>
       </c>
       <c r="D8" t="n">
-        <v>11.6</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="9">
@@ -7859,13 +7843,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>252038</v>
+        <v>254465</v>
       </c>
       <c r="C9" t="n">
-        <v>21445</v>
+        <v>24317</v>
       </c>
       <c r="D9" t="n">
-        <v>8.5</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="10">
@@ -7875,13 +7859,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>278028</v>
+        <v>280295</v>
       </c>
       <c r="C10" t="n">
-        <v>39063</v>
+        <v>41188</v>
       </c>
       <c r="D10" t="n">
-        <v>14.1</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="11">
@@ -7891,13 +7875,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>274224</v>
+        <v>276618</v>
       </c>
       <c r="C11" t="n">
-        <v>30476</v>
+        <v>33111</v>
       </c>
       <c r="D11" t="n">
-        <v>11.1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -7907,13 +7891,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>273239</v>
+        <v>275370</v>
       </c>
       <c r="C12" t="n">
-        <v>26768</v>
+        <v>29080</v>
       </c>
       <c r="D12" t="n">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
     </row>
   </sheetData>
@@ -7959,13 +7943,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>383154</v>
+        <v>386306</v>
       </c>
       <c r="C2" t="n">
-        <v>36882</v>
+        <v>40361</v>
       </c>
       <c r="D2" t="n">
-        <v>9.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="3">
@@ -7975,13 +7959,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>145697</v>
+        <v>146725</v>
       </c>
       <c r="C3" t="n">
-        <v>17252</v>
+        <v>18525</v>
       </c>
       <c r="D3" t="n">
-        <v>11.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="4">
@@ -7991,13 +7975,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>146585</v>
+        <v>148031</v>
       </c>
       <c r="C4" t="n">
-        <v>16674</v>
+        <v>18243</v>
       </c>
       <c r="D4" t="n">
-        <v>11.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="5">
@@ -8007,13 +7991,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150106</v>
+        <v>150889</v>
       </c>
       <c r="C5" t="n">
-        <v>16205</v>
+        <v>17128</v>
       </c>
       <c r="D5" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="6">
@@ -8023,13 +8007,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150578</v>
+        <v>151895</v>
       </c>
       <c r="C6" t="n">
-        <v>13353</v>
+        <v>14587</v>
       </c>
       <c r="D6" t="n">
-        <v>8.9</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="7">
@@ -8039,13 +8023,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>128979</v>
+        <v>129799</v>
       </c>
       <c r="C7" t="n">
-        <v>10635</v>
+        <v>11550</v>
       </c>
       <c r="D7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="8">
@@ -8055,13 +8039,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>86216</v>
+        <v>86819</v>
       </c>
       <c r="C8" t="n">
-        <v>9613</v>
+        <v>10212</v>
       </c>
       <c r="D8" t="n">
-        <v>11.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="9">
@@ -8071,13 +8055,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>83257</v>
+        <v>84105</v>
       </c>
       <c r="C9" t="n">
-        <v>6762</v>
+        <v>7836</v>
       </c>
       <c r="D9" t="n">
-        <v>8.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -8087,13 +8071,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55646</v>
+        <v>56069</v>
       </c>
       <c r="C10" t="n">
-        <v>6573</v>
+        <v>6997</v>
       </c>
       <c r="D10" t="n">
-        <v>11.8</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="11">
@@ -8103,13 +8087,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>74859</v>
+        <v>75402</v>
       </c>
       <c r="C11" t="n">
-        <v>6322</v>
+        <v>6908</v>
       </c>
       <c r="D11" t="n">
-        <v>8.4</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -8119,13 +8103,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>54521</v>
+        <v>54899</v>
       </c>
       <c r="C12" t="n">
-        <v>6304</v>
+        <v>6655</v>
       </c>
       <c r="D12" t="n">
-        <v>11.6</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="13">
@@ -8135,13 +8119,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>50574</v>
+        <v>50804</v>
       </c>
       <c r="C13" t="n">
-        <v>6265</v>
+        <v>6557</v>
       </c>
       <c r="D13" t="n">
-        <v>12.4</v>
+        <v>12.9</v>
       </c>
     </row>
   </sheetData>
@@ -8197,13 +8181,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>96641</v>
+        <v>102536</v>
       </c>
       <c r="D2" t="n">
-        <v>21745</v>
+        <v>28866</v>
       </c>
       <c r="E2" t="n">
-        <v>22.5</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="3">
@@ -8218,13 +8202,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65350</v>
+        <v>72492</v>
       </c>
       <c r="D3" t="n">
-        <v>18388</v>
+        <v>25235</v>
       </c>
       <c r="E3" t="n">
-        <v>28.1</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="4">
@@ -8239,13 +8223,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>190374</v>
+        <v>193393</v>
       </c>
       <c r="D4" t="n">
-        <v>27363</v>
+        <v>29599</v>
       </c>
       <c r="E4" t="n">
-        <v>14.4</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="5">
@@ -8260,13 +8244,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>119543</v>
+        <v>123011</v>
       </c>
       <c r="D5" t="n">
-        <v>26475</v>
+        <v>28277</v>
       </c>
       <c r="E5" t="n">
-        <v>22.1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -8281,13 +8265,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>259795</v>
+        <v>261883</v>
       </c>
       <c r="D6" t="n">
-        <v>29202</v>
+        <v>30953</v>
       </c>
       <c r="E6" t="n">
-        <v>11.2</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="7">
@@ -8302,13 +8286,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>176526</v>
+        <v>180211</v>
       </c>
       <c r="D7" t="n">
-        <v>28682</v>
+        <v>30326</v>
       </c>
       <c r="E7" t="n">
-        <v>16.2</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="8">
@@ -8323,13 +8307,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>268647</v>
+        <v>270719</v>
       </c>
       <c r="D8" t="n">
-        <v>25566</v>
+        <v>26717</v>
       </c>
       <c r="E8" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="9">
@@ -8344,13 +8328,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>216755</v>
+        <v>219253</v>
       </c>
       <c r="D9" t="n">
-        <v>27334</v>
+        <v>28669</v>
       </c>
       <c r="E9" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="10">
@@ -8365,13 +8349,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>301690</v>
+        <v>303499</v>
       </c>
       <c r="D10" t="n">
-        <v>24283</v>
+        <v>25395</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="11">
@@ -8386,13 +8370,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>311627</v>
+        <v>315686</v>
       </c>
       <c r="D11" t="n">
-        <v>29665</v>
+        <v>31411</v>
       </c>
       <c r="E11" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -8407,13 +8391,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>301687</v>
+        <v>304215</v>
       </c>
       <c r="D12" t="n">
-        <v>18361</v>
+        <v>19344</v>
       </c>
       <c r="E12" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="13">
@@ -8428,13 +8412,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>298970</v>
+        <v>305598</v>
       </c>
       <c r="D13" t="n">
-        <v>20611</v>
+        <v>22225</v>
       </c>
       <c r="E13" t="n">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="14">
@@ -8449,13 +8433,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>213515</v>
+        <v>219357</v>
       </c>
       <c r="D14" t="n">
-        <v>11680</v>
+        <v>12383</v>
       </c>
       <c r="E14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="15">
@@ -8470,13 +8454,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>219647</v>
+        <v>226553</v>
       </c>
       <c r="D15" t="n">
-        <v>13964</v>
+        <v>14924</v>
       </c>
       <c r="E15" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="16">
@@ -8491,13 +8475,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1263</v>
+        <v>1848</v>
       </c>
       <c r="D16" t="n">
-        <v>1261</v>
+        <v>1847</v>
       </c>
       <c r="E16" t="n">
-        <v>99.8</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -8512,10 +8496,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>802</v>
+        <v>1542</v>
       </c>
       <c r="D17" t="n">
-        <v>802</v>
+        <v>1542</v>
       </c>
       <c r="E17" t="n">
         <v>100</v>
@@ -8583,10 +8567,10 @@
         <v>28.7</v>
       </c>
       <c r="E2" t="n">
-        <v>33.5</v>
+        <v>32</v>
       </c>
       <c r="F2" t="n">
-        <v>-4.8</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="3">
@@ -8605,10 +8589,10 @@
         <v>32.2</v>
       </c>
       <c r="E3" t="n">
-        <v>34.5</v>
+        <v>34.1</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.3</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="4">
@@ -8627,10 +8611,10 @@
         <v>44.5</v>
       </c>
       <c r="E4" t="n">
-        <v>46.9</v>
+        <v>46.4</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.4</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="5">
@@ -8649,10 +8633,10 @@
         <v>54.1</v>
       </c>
       <c r="E5" t="n">
-        <v>57.3</v>
+        <v>57</v>
       </c>
       <c r="F5" t="n">
-        <v>-3.2</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="6">
@@ -8671,10 +8655,10 @@
         <v>63.9</v>
       </c>
       <c r="E6" t="n">
-        <v>65.59999999999999</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.7</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="7">
@@ -8715,10 +8699,10 @@
         <v>68.09999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>70</v>
+        <v>70.5</v>
       </c>
       <c r="F8" t="n">
-        <v>-1.9</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="9">
@@ -8796,13 +8780,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>96641</v>
+        <v>102536</v>
       </c>
       <c r="D2" t="n">
-        <v>401416</v>
+        <v>414587</v>
       </c>
       <c r="E2" t="n">
-        <v>24.1</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="3">
@@ -8817,13 +8801,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65350</v>
+        <v>72492</v>
       </c>
       <c r="D3" t="n">
-        <v>222665</v>
+        <v>237358</v>
       </c>
       <c r="E3" t="n">
-        <v>29.3</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="4">
@@ -8838,13 +8822,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>190374</v>
+        <v>193393</v>
       </c>
       <c r="D4" t="n">
-        <v>710623</v>
+        <v>728719</v>
       </c>
       <c r="E4" t="n">
-        <v>26.8</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="5">
@@ -8859,13 +8843,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>119543</v>
+        <v>123011</v>
       </c>
       <c r="D5" t="n">
-        <v>383245</v>
+        <v>396490</v>
       </c>
       <c r="E5" t="n">
-        <v>31.2</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -8880,13 +8864,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>259795</v>
+        <v>261883</v>
       </c>
       <c r="D6" t="n">
-        <v>657930</v>
+        <v>670055</v>
       </c>
       <c r="E6" t="n">
-        <v>39.5</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="7">
@@ -8901,13 +8885,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>176526</v>
+        <v>180211</v>
       </c>
       <c r="D7" t="n">
-        <v>406600</v>
+        <v>418598</v>
       </c>
       <c r="E7" t="n">
-        <v>43.4</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="8">
@@ -8922,13 +8906,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>268647</v>
+        <v>270719</v>
       </c>
       <c r="D8" t="n">
-        <v>541152</v>
+        <v>548477</v>
       </c>
       <c r="E8" t="n">
-        <v>49.6</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="9">
@@ -8943,13 +8927,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>216755</v>
+        <v>219253</v>
       </c>
       <c r="D9" t="n">
-        <v>404558</v>
+        <v>411833</v>
       </c>
       <c r="E9" t="n">
-        <v>53.6</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="10">
@@ -8964,13 +8948,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>301690</v>
+        <v>303499</v>
       </c>
       <c r="D10" t="n">
-        <v>516154</v>
+        <v>520500</v>
       </c>
       <c r="E10" t="n">
-        <v>58.4</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="11">
@@ -8985,13 +8969,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>311627</v>
+        <v>315686</v>
       </c>
       <c r="D11" t="n">
-        <v>487137</v>
+        <v>494722</v>
       </c>
       <c r="E11" t="n">
-        <v>64</v>
+        <v>63.8</v>
       </c>
     </row>
     <row r="12">
@@ -9006,13 +8990,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>301687</v>
+        <v>304215</v>
       </c>
       <c r="D12" t="n">
-        <v>447622</v>
+        <v>450944</v>
       </c>
       <c r="E12" t="n">
-        <v>67.40000000000001</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="13">
@@ -9027,13 +9011,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>298970</v>
+        <v>305598</v>
       </c>
       <c r="D13" t="n">
-        <v>417546</v>
+        <v>426306</v>
       </c>
       <c r="E13" t="n">
-        <v>71.59999999999999</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="14">
@@ -9048,13 +9032,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>213515</v>
+        <v>219357</v>
       </c>
       <c r="D14" t="n">
-        <v>337484</v>
+        <v>341197</v>
       </c>
       <c r="E14" t="n">
-        <v>63.3</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="15">
@@ -9069,13 +9053,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>219647</v>
+        <v>226553</v>
       </c>
       <c r="D15" t="n">
-        <v>331780</v>
+        <v>336885</v>
       </c>
       <c r="E15" t="n">
-        <v>66.2</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="16">
@@ -9090,13 +9074,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1263</v>
+        <v>1848</v>
       </c>
       <c r="D16" t="n">
-        <v>10343</v>
+        <v>9626</v>
       </c>
       <c r="E16" t="n">
-        <v>12.2</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="17">
@@ -9111,13 +9095,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>802</v>
+        <v>1542</v>
       </c>
       <c r="D17" t="n">
-        <v>5711</v>
+        <v>5999</v>
       </c>
       <c r="E17" t="n">
-        <v>14</v>
+        <v>25.7</v>
       </c>
     </row>
   </sheetData>
@@ -9182,10 +9166,10 @@
         <v>52.8</v>
       </c>
       <c r="E2" t="n">
-        <v>55.4</v>
+        <v>55.1</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.6</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="3">
@@ -9204,10 +9188,10 @@
         <v>50.8</v>
       </c>
       <c r="E3" t="n">
-        <v>52</v>
+        <v>51.6</v>
       </c>
       <c r="F3" t="n">
-        <v>-1.2</v>
+        <v>-0.8</v>
       </c>
     </row>
   </sheetData>
@@ -9246,10 +9230,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>61556</v>
+        <v>86682</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="3">
@@ -9257,10 +9241,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>224079</v>
+        <v>224150</v>
       </c>
       <c r="C3" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="4">
@@ -9268,10 +9252,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>452566</v>
+        <v>452628</v>
       </c>
       <c r="C4" t="n">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="5">
@@ -9279,10 +9263,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>594794</v>
+        <v>594892</v>
       </c>
       <c r="C5" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="6">
@@ -9290,10 +9274,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1743423</v>
+        <v>1743457</v>
       </c>
       <c r="C6" t="n">
-        <v>56.7</v>
+        <v>56.2</v>
       </c>
     </row>
   </sheetData>
@@ -9537,16 +9521,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>557525</v>
+        <v>562319</v>
       </c>
       <c r="C2" t="n">
-        <v>229022</v>
+        <v>230690</v>
       </c>
       <c r="D2" t="n">
-        <v>2404</v>
+        <v>2421</v>
       </c>
       <c r="E2" t="n">
-        <v>844661</v>
+        <v>862020</v>
       </c>
     </row>
     <row r="3">
@@ -9556,16 +9540,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>505008</v>
+        <v>513769</v>
       </c>
       <c r="C3" t="n">
-        <v>85194</v>
+        <v>86535</v>
       </c>
       <c r="D3" t="n">
-        <v>1847</v>
+        <v>1898</v>
       </c>
       <c r="E3" t="n">
-        <v>817171</v>
+        <v>842144</v>
       </c>
     </row>
     <row r="4">
@@ -9575,16 +9559,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13592</v>
+        <v>37</v>
       </c>
       <c r="C4" t="n">
-        <v>3018</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
         <v>69</v>
-      </c>
-      <c r="E4" t="n">
-        <v>42401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>